<commit_message>
feat: refresh report pipeline configuration
</commit_message>
<xml_diff>
--- a/scripts/房地产-半自动化表格.xlsx
+++ b/scripts/房地产-半自动化表格.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucius\Desktop\asset_mgnt_report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucius\Desktop\asset_mgnt_report\codex\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25CBE280-83A6-4295-8874-34CC195D6A0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0514DA7C-FF72-43FE-B014-7BD9078C1F86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" tabRatio="784" xr2:uid="{D1DDF7B5-99D9-344F-819C-1A690CDC6D20}"/>
   </bookViews>
@@ -27,11 +27,11 @@
     <sheet name="rawData_RentPriceIndex_US" sheetId="7" r:id="rId12"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_1" localSheetId="3" hidden="1">Processed_HousePriceIndex_CN_HK!$A$1:$L$71</definedName>
-    <definedName name="ExternalData_1" localSheetId="4" hidden="1">Processed_HousePriceIndex_US_CA!$A$1:$L$70</definedName>
-    <definedName name="ExternalData_1" localSheetId="6" hidden="1">Processed_RentPrice_US_CA!$A$1:$L$70</definedName>
-    <definedName name="ExternalData_2" localSheetId="2" hidden="1">Processed_HousePriceIndex_CN_SZ!$A$1:$L$73</definedName>
-    <definedName name="ExternalData_2" localSheetId="5" hidden="1">'Processed_RentPrice_CN_HK '!$A$1:$L$71</definedName>
+    <definedName name="ExternalData_1" localSheetId="3" hidden="1">Processed_HousePriceIndex_CN_HK!$A$1:$L$77</definedName>
+    <definedName name="ExternalData_1" localSheetId="4" hidden="1">Processed_HousePriceIndex_US_CA!$A$1:$L$76</definedName>
+    <definedName name="ExternalData_1" localSheetId="6" hidden="1">Processed_RentPrice_US_CA!$A$1:$L$77</definedName>
+    <definedName name="ExternalData_2" localSheetId="2" hidden="1">Processed_HousePriceIndex_CN_SZ!$A$1:$L$79</definedName>
+    <definedName name="ExternalData_2" localSheetId="5" hidden="1">'Processed_RentPrice_CN_HK '!$A$1:$L$77</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -99,7 +99,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1441" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1543" uniqueCount="65">
   <si>
     <t>上月=100</t>
   </si>
@@ -508,7 +508,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="11">
+  <numFmts count="12">
     <numFmt numFmtId="176" formatCode="yyyy/mm/dd"/>
     <numFmt numFmtId="177" formatCode="yyyy/mm"/>
     <numFmt numFmtId="178" formatCode="0.00_ "/>
@@ -520,6 +520,7 @@
     <numFmt numFmtId="184" formatCode="0_ "/>
     <numFmt numFmtId="185" formatCode="#,##0_ "/>
     <numFmt numFmtId="186" formatCode="#,##0.00_ "/>
+    <numFmt numFmtId="187" formatCode="0.000_ "/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -816,7 +817,7 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -921,6 +922,34 @@
     <xf numFmtId="185" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="177" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="177" fontId="15" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="187" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -953,33 +982,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="2" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="177" fontId="15" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1303,8 +1305,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{2E01295C-C38B-984E-843D-A42CD6AA8A28}" name="Processed_CN_SZ" displayName="Processed_CN_SZ" ref="A1:N73" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:N73" xr:uid="{2E01295C-C38B-984E-843D-A42CD6AA8A28}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{2E01295C-C38B-984E-843D-A42CD6AA8A28}" name="Processed_CN_SZ" displayName="Processed_CN_SZ" ref="A1:N79" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:N79" xr:uid="{2E01295C-C38B-984E-843D-A42CD6AA8A28}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{064CA3F1-611E-6E4D-BA50-4AB6879EDABD}" uniqueName="1" name="Date" queryTableFieldId="1" dataDxfId="48"/>
     <tableColumn id="2" xr3:uid="{665CBE8E-9DF2-524E-91B7-129CDF2653E0}" uniqueName="2" name="Value" queryTableFieldId="2" dataDxfId="47"/>
@@ -1330,8 +1332,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A668228E-8AFE-6949-B93A-9E80E041B773}" name="Processed_CN_HK" displayName="Processed_CN_HK" ref="A1:N71" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:N71" xr:uid="{A668228E-8AFE-6949-B93A-9E80E041B773}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A668228E-8AFE-6949-B93A-9E80E041B773}" name="Processed_CN_HK" displayName="Processed_CN_HK" ref="A1:N77" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:N77" xr:uid="{A668228E-8AFE-6949-B93A-9E80E041B773}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{D1E59232-7D95-EB40-BDED-271655203721}" uniqueName="1" name="Date" queryTableFieldId="1" dataDxfId="38"/>
     <tableColumn id="2" xr3:uid="{2D53112B-D659-A242-9E60-601A62778041}" uniqueName="2" name="Value" queryTableFieldId="2" dataDxfId="37"/>
@@ -1357,8 +1359,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{345E0904-0077-5C4F-8D1D-BD5DB0E8300A}" name="Processed_US_CA" displayName="Processed_US_CA" ref="A1:N70" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:N70" xr:uid="{345E0904-0077-5C4F-8D1D-BD5DB0E8300A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{345E0904-0077-5C4F-8D1D-BD5DB0E8300A}" name="Processed_US_CA" displayName="Processed_US_CA" ref="A1:N76" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:N76" xr:uid="{345E0904-0077-5C4F-8D1D-BD5DB0E8300A}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{839ECA1F-FCB2-CE49-909D-BEF917E29F4C}" uniqueName="1" name="Date" queryTableFieldId="1" dataDxfId="29"/>
     <tableColumn id="2" xr3:uid="{ED9CE58E-DF97-0143-85D3-BD189E485C22}" uniqueName="2" name="Value" queryTableFieldId="2" dataDxfId="28"/>
@@ -1384,8 +1386,8 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{EEA05C33-CE2D-DD44-B4CD-86EE7617844E}" name="Processed_RentPrice_CN_HK__2" displayName="Processed_RentPrice_CN_HK__2" ref="A1:N71" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:N71" xr:uid="{EEA05C33-CE2D-DD44-B4CD-86EE7617844E}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{EEA05C33-CE2D-DD44-B4CD-86EE7617844E}" name="Processed_RentPrice_CN_HK__2" displayName="Processed_RentPrice_CN_HK__2" ref="A1:N77" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:N77" xr:uid="{EEA05C33-CE2D-DD44-B4CD-86EE7617844E}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{3130BF33-BE82-C04F-A72F-C84B593F86FA}" uniqueName="1" name="Date" queryTableFieldId="1" dataDxfId="18"/>
     <tableColumn id="2" xr3:uid="{2E5D16A7-E903-1E44-AB24-5C76F52C87CD}" uniqueName="2" name="Value" queryTableFieldId="2" dataDxfId="17"/>
@@ -1411,8 +1413,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{5BB058DC-488B-574D-889C-352D3A8E1EEA}" name="Processed_RentPrice_US_CA__2" displayName="Processed_RentPrice_US_CA__2" ref="A1:N70" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:N70" xr:uid="{5BB058DC-488B-574D-889C-352D3A8E1EEA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{5BB058DC-488B-574D-889C-352D3A8E1EEA}" name="Processed_RentPrice_US_CA__2" displayName="Processed_RentPrice_US_CA__2" ref="A1:N77" tableType="queryTable" totalsRowShown="0">
+  <autoFilter ref="A1:N77" xr:uid="{5BB058DC-488B-574D-889C-352D3A8E1EEA}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{480AB120-2152-2440-BC03-EB6C8B2EDED7}" uniqueName="1" name="Date" queryTableFieldId="1" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{592A00D3-04E6-094F-ADBE-1BEB0F9429F6}" uniqueName="2" name="Value" queryTableFieldId="2"/>
@@ -1758,10 +1760,10 @@
   <sheetFormatPr defaultColWidth="10.78125" defaultRowHeight="27.5"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="44" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="52"/>
+      <c r="B1" s="45"/>
       <c r="C1" s="12" t="s">
         <v>6</v>
       </c>
@@ -1773,25 +1775,25 @@
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="56" t="s">
+      <c r="A2" s="48" t="s">
         <v>64</v>
       </c>
-      <c r="B2" s="57"/>
-      <c r="C2" s="58">
+      <c r="B2" s="49"/>
+      <c r="C2" s="40">
         <f>_xlfn.XLOOKUP(MAX(Processed_CN_SZ[Date]), Processed_CN_SZ[Date], Processed_CN_SZ[Date])</f>
-        <v>45992</v>
-      </c>
-      <c r="D2" s="58">
+        <v>46174</v>
+      </c>
+      <c r="D2" s="40">
         <f>_xlfn.XLOOKUP(MAX(Processed_CN_HK[Date]), Processed_CN_HK[Date], Processed_CN_HK[Date])</f>
-        <v>45931</v>
-      </c>
-      <c r="E2" s="59">
+        <v>46113</v>
+      </c>
+      <c r="E2" s="41">
         <f>_xlfn.XLOOKUP(MAX(Processed_US_CA[Date]), Processed_US_CA[Date], Processed_US_CA[Date])</f>
-        <v>45901</v>
+        <v>46082</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="46" t="s">
+      <c r="A3" s="56" t="s">
         <v>9</v>
       </c>
       <c r="B3" s="3" t="s">
@@ -1799,109 +1801,109 @@
       </c>
       <c r="C3" s="23" cm="1">
         <f t="array" ref="C3">ROUND(_xlfn.XLOOKUP(MAX(Processed_CN_SZ[Date]), Processed_CN_SZ[Date], Processed_CN_SZ[Value]) / AVERAGE(_xlfn._xlws.FILTER(Processed_CN_SZ[Value], YEAR(Processed_CN_SZ[Date])=2020)), 3) * 100</f>
-        <v>96</v>
+        <v>93.600000000000009</v>
       </c>
       <c r="D3" s="23" cm="1">
         <f t="array" ref="D3">ROUND(_xlfn.XLOOKUP(MAX(Processed_CN_HK[Date]), Processed_CN_HK[Date], Processed_CN_HK[Value]) / AVERAGE(_xlfn._xlws.FILTER(Processed_CN_HK[Value], YEAR(Processed_CN_HK[Date])=2020)), 3) * 100</f>
-        <v>77.2</v>
+        <v>83.1</v>
       </c>
       <c r="E3" s="24" cm="1">
         <f t="array" ref="E3">ROUND(_xlfn.XLOOKUP(MAX(Processed_US_CA[Date]), Processed_US_CA[Date], Processed_US_CA[Value]) / AVERAGE(_xlfn._xlws.FILTER(Processed_US_CA[Value], YEAR(Processed_US_CA[Date])=2020)), 3) * 100</f>
-        <v>127.2</v>
+        <v>129.1</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="47"/>
+      <c r="A4" s="57"/>
       <c r="B4" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C4" s="25">
         <f>_xlfn.XLOOKUP(MAX(Processed_CN_SZ[Date]), Processed_CN_SZ[Date], Processed_CN_SZ[上月=100])</f>
-        <v>99.739491263653449</v>
+        <v>99.746115374336654</v>
       </c>
       <c r="D4" s="25">
         <f>_xlfn.XLOOKUP(MAX(Processed_CN_HK[Date]), Processed_CN_HK[Date], Processed_CN_HK[上月=100])</f>
-        <v>100.40941658137154</v>
+        <v>101.21483375959079</v>
       </c>
       <c r="E4" s="26">
         <f>_xlfn.XLOOKUP(MAX(Processed_US_CA[Date]), Processed_US_CA[Date], Processed_US_CA[上月=100])</f>
-        <v>100.87515846081257</v>
+        <v>99.643246187418839</v>
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="47"/>
+      <c r="A5" s="57"/>
       <c r="B5" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C5" s="25">
         <f>_xlfn.XLOOKUP(MAX(Processed_CN_SZ[Date]), Processed_CN_SZ[Date], Processed_CN_SZ[上年同月=100])</f>
-        <v>91.627207302688944</v>
+        <v>91.736306179775283</v>
       </c>
       <c r="D5" s="25">
         <f>_xlfn.XLOOKUP(MAX(Processed_CN_HK[Date]), Processed_CN_HK[Date], Processed_CN_HK[上年同月=100])</f>
-        <v>101.13402061855669</v>
+        <v>110.50610820244329</v>
       </c>
       <c r="E5" s="26">
         <f>_xlfn.XLOOKUP(MAX(Processed_US_CA[Date]), Processed_US_CA[Date], Processed_US_CA[上年同月=100])</f>
-        <v>99.075963608041079</v>
+        <v>100.47197258480809</v>
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="47"/>
+      <c r="A6" s="57"/>
       <c r="B6" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C6" s="27">
         <f>_xlfn.XLOOKUP(MAX(Processed_CN_SZ[Date]), Processed_CN_SZ[Date], Processed_CN_SZ[YoY])</f>
-        <v>-8.3727926973110656E-2</v>
+        <v>-8.2636938202247184E-2</v>
       </c>
       <c r="D6" s="27">
         <f>_xlfn.XLOOKUP(MAX(Processed_CN_HK[Date]), Processed_CN_HK[Date], Processed_CN_HK[YoY])</f>
-        <v>1.134020618556705E-2</v>
+        <v>0.10506108202443289</v>
       </c>
       <c r="E6" s="28">
         <f>_xlfn.XLOOKUP(MAX(Processed_US_CA[Date]), Processed_US_CA[Date], Processed_US_CA[YoY])</f>
-        <v>-9.2403639195892985E-3</v>
+        <v>4.7197258480809754E-3</v>
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="47"/>
+      <c r="A7" s="57"/>
       <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C7" s="27">
         <f>_xlfn.XLOOKUP(MAX(Processed_CN_SZ[Date]), Processed_CN_SZ[Date], Processed_CN_SZ[MoM])</f>
-        <v>-2.6050873634655106E-3</v>
+        <v>-2.5388462566334519E-3</v>
       </c>
       <c r="D7" s="27">
         <f>_xlfn.XLOOKUP(MAX(Processed_CN_HK[Date]), Processed_CN_HK[Date], Processed_CN_HK[MoM])</f>
-        <v>4.0941658137154165E-3</v>
+        <v>1.2148337595907964E-2</v>
       </c>
       <c r="E7" s="28">
         <f>_xlfn.XLOOKUP(MAX(Processed_US_CA[Date]), Processed_US_CA[Date], Processed_US_CA[MoM])</f>
-        <v>8.7515846081257214E-3</v>
+        <v>-3.567538125811578E-3</v>
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="48"/>
+      <c r="A8" s="58"/>
       <c r="B8" s="2" t="s">
         <v>4</v>
       </c>
       <c r="C8" s="27">
         <f>_xlfn.XLOOKUP(MAX(Processed_CN_SZ[Date]), Processed_CN_SZ[Date], Processed_CN_SZ[YTD(%)])</f>
-        <v>-8.4025428073413289E-2</v>
+        <v>-2.1296122869451262E-2</v>
       </c>
       <c r="D8" s="27">
         <f>_xlfn.XLOOKUP(MAX(Processed_CN_HK[Date]), Processed_CN_HK[Date], Processed_CN_HK[YTD(%)])</f>
-        <v>2.4721448467966756E-2</v>
+        <v>4.488448844884485E-2</v>
       </c>
       <c r="E8" s="28">
         <f>_xlfn.XLOOKUP(MAX(Processed_US_CA[Date]), Processed_US_CA[Date], Processed_US_CA[YTD(%)])</f>
-        <v>-2.2542868631674096E-2</v>
+        <v>-2.2773766335568713E-3</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="46" t="s">
+      <c r="A9" s="56" t="s">
         <v>12</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -1912,15 +1914,15 @@
       </c>
       <c r="D9" s="23" cm="1">
         <f t="array" ref="D9">ROUND(_xlfn.XLOOKUP(MAX(Processed_RentPrice_CN_HK__2[Date]), Processed_RentPrice_CN_HK__2[Date], Processed_RentPrice_CN_HK__2[Value]) / AVERAGE(_xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Value], YEAR(Processed_RentPrice_CN_HK__2[Date])=2020)), 3) * 100</f>
-        <v>111.00000000000001</v>
+        <v>112.79999999999998</v>
       </c>
       <c r="E9" s="24" cm="1">
         <f t="array" ref="E9">ROUND(_xlfn.XLOOKUP(MAX(Processed_RentPrice_US_CA__2[Date]), Processed_RentPrice_US_CA__2[Date], Processed_RentPrice_US_CA__2[Value]) / AVERAGE(_xlfn._xlws.FILTER(Processed_RentPrice_US_CA__2[Value], YEAR(Processed_RentPrice_US_CA__2[Date])=2020)), 3) * 100</f>
-        <v>111.60000000000001</v>
+        <v>113.9</v>
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="47"/>
+      <c r="A10" s="57"/>
       <c r="B10" s="1" t="s">
         <v>10</v>
       </c>
@@ -1929,16 +1931,16 @@
       </c>
       <c r="D10" s="25">
         <f>_xlfn.XLOOKUP(MAX(Processed_RentPrice_CN_HK__2[Date]), Processed_RentPrice_CN_HK__2[Date], Processed_RentPrice_CN_HK__2[上月=100])</f>
-        <v>100</v>
+        <v>100.59347181008901</v>
       </c>
       <c r="E10" s="26">
         <f>_xlfn.XLOOKUP(MAX(Processed_RentPrice_US_CA__2[Date]), Processed_RentPrice_US_CA__2[Date], Processed_RentPrice_US_CA__2[上月=100])</f>
-        <v>100.2378205867651</v>
+        <v>100.75850094765282</v>
       </c>
       <c r="F10" s="4"/>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="47"/>
+      <c r="A11" s="57"/>
       <c r="B11" s="1" t="s">
         <v>11</v>
       </c>
@@ -1947,15 +1949,15 @@
       </c>
       <c r="D11" s="25">
         <f>_xlfn.XLOOKUP(MAX(Processed_RentPrice_CN_HK__2[Date]), Processed_RentPrice_CN_HK__2[Date], Processed_RentPrice_CN_HK__2[上年同月=100])</f>
-        <v>103.89206019719772</v>
+        <v>104.89943269726663</v>
       </c>
       <c r="E11" s="26">
         <f>_xlfn.XLOOKUP(MAX(Processed_RentPrice_US_CA__2[Date]), Processed_RentPrice_US_CA__2[Date], Processed_RentPrice_US_CA__2[上年同月=100])</f>
-        <v>102.11005419082926</v>
+        <v>102.65970376143498</v>
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="47"/>
+      <c r="A12" s="57"/>
       <c r="B12" s="1" t="s">
         <v>2</v>
       </c>
@@ -1964,15 +1966,15 @@
       </c>
       <c r="D12" s="27">
         <f>_xlfn.XLOOKUP(MAX(Processed_RentPrice_CN_HK__2[Date]), Processed_RentPrice_CN_HK__2[Date], Processed_RentPrice_CN_HK__2[YoY])</f>
-        <v>3.8920601971977171E-2</v>
+        <v>4.899432697266632E-2</v>
       </c>
       <c r="E12" s="28">
         <f>_xlfn.XLOOKUP(MAX(Processed_RentPrice_US_CA__2[Date]), Processed_RentPrice_US_CA__2[Date], Processed_RentPrice_US_CA__2[YoY])</f>
-        <v>2.1100541908292633E-2</v>
+        <v>2.6597037614349773E-2</v>
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="47"/>
+      <c r="A13" s="57"/>
       <c r="B13" s="1" t="s">
         <v>3</v>
       </c>
@@ -1981,15 +1983,15 @@
       </c>
       <c r="D13" s="27">
         <f>_xlfn.XLOOKUP(MAX(Processed_RentPrice_CN_HK__2[Date]), Processed_RentPrice_CN_HK__2[Date], Processed_RentPrice_CN_HK__2[MoM])</f>
-        <v>0</v>
+        <v>5.9347181008902921E-3</v>
       </c>
       <c r="E13" s="28">
         <f>_xlfn.XLOOKUP(MAX(Processed_RentPrice_US_CA__2[Date]), Processed_RentPrice_US_CA__2[Date], Processed_RentPrice_US_CA__2[MoM])</f>
-        <v>2.3782058676509524E-3</v>
+        <v>7.5850094765282606E-3</v>
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="48"/>
+      <c r="A14" s="58"/>
       <c r="B14" s="17" t="s">
         <v>4</v>
       </c>
@@ -1998,86 +2000,86 @@
       </c>
       <c r="D14" s="27">
         <f>_xlfn.XLOOKUP(MAX(Processed_RentPrice_CN_HK__2[Date]), Processed_RentPrice_CN_HK__2[Date], Processed_RentPrice_CN_HK__2[YTD(%)])</f>
-        <v>3.8381742738589075E-2</v>
+        <v>1.294820717131473E-2</v>
       </c>
       <c r="E14" s="28">
         <f>_xlfn.XLOOKUP(MAX(Processed_RentPrice_US_CA__2[Date]), Processed_RentPrice_US_CA__2[Date], Processed_RentPrice_US_CA__2[YTD(%)])</f>
-        <v>7.3341177516175193E-3</v>
+        <v>1.0930871829163857E-2</v>
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="49" t="s">
+      <c r="A15" s="59" t="s">
         <v>49</v>
       </c>
-      <c r="B15" s="50"/>
+      <c r="B15" s="60"/>
       <c r="C15" s="27" t="s">
         <v>39</v>
       </c>
       <c r="D15" s="38">
         <f>'price-to-rent ratio'!H3</f>
-        <v>149679</v>
+        <v>182317</v>
       </c>
       <c r="E15" s="39">
         <f>'price-to-rent ratio'!I3</f>
-        <v>1255433</v>
+        <v>1369171</v>
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="49" t="s">
+      <c r="A16" s="59" t="s">
         <v>50</v>
       </c>
-      <c r="B16" s="50"/>
+      <c r="B16" s="60"/>
       <c r="C16" s="37" t="s">
         <v>39</v>
       </c>
       <c r="D16" s="38">
         <f>'price-to-rent ratio'!H6</f>
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="E16" s="39">
         <f>'price-to-rent ratio'!I6</f>
-        <v>3587</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="17" spans="1:5">
-      <c r="A17" s="49" t="s">
+      <c r="A17" s="59" t="s">
         <v>51</v>
       </c>
-      <c r="B17" s="50"/>
+      <c r="B17" s="60"/>
       <c r="C17" s="27">
         <f>'price-to-rent ratio'!G7</f>
-        <v>1.9736335985847293E-2</v>
+        <v>1.9534038537971699E-2</v>
       </c>
       <c r="D17" s="27">
         <f>'price-to-rent ratio'!H7</f>
-        <v>3.3191028801635498E-2</v>
+        <v>2.770997767624522E-2</v>
       </c>
       <c r="E17" s="28">
         <f>'price-to-rent ratio'!I7</f>
-        <v>3.4286178553534913E-2</v>
+        <v>3.5057710103412944E-2</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="27.5" customHeight="1">
-      <c r="A18" s="51" t="s">
+      <c r="A18" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="52"/>
-      <c r="C18" s="44" t="s">
+      <c r="B18" s="45"/>
+      <c r="C18" s="54" t="s">
         <v>43</v>
       </c>
-      <c r="D18" s="40" t="s">
+      <c r="D18" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="E18" s="42" t="s">
+      <c r="E18" s="52" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:5">
-      <c r="A19" s="53"/>
-      <c r="B19" s="54"/>
-      <c r="C19" s="45"/>
-      <c r="D19" s="41"/>
-      <c r="E19" s="43"/>
+      <c r="A19" s="46"/>
+      <c r="B19" s="47"/>
+      <c r="C19" s="55"/>
+      <c r="D19" s="51"/>
+      <c r="E19" s="53"/>
     </row>
     <row r="20" spans="1:5" ht="27.5" customHeight="1"/>
   </sheetData>
@@ -2102,7 +2104,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0C340C42-17FD-A344-A336-548598A6372C}">
-  <dimension ref="A1:E70"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr defaultColWidth="10.78125" defaultRowHeight="27.5"/>
   <cols>
     <col min="2" max="2" width="10.5625" style="11" customWidth="1"/>
@@ -3201,8 +3203,8 @@
       <c r="A65" s="6">
         <v>45748</v>
       </c>
-      <c r="B65" s="15">
-        <v>354.17</v>
+      <c r="B65" s="42">
+        <v>354.19372711900598</v>
       </c>
       <c r="C65" t="s">
         <v>37</v>
@@ -3218,8 +3220,8 @@
       <c r="A66" s="6">
         <v>45778</v>
       </c>
-      <c r="B66" s="15">
-        <v>351.71199999999999</v>
+      <c r="B66" s="42">
+        <v>352.11270457490201</v>
       </c>
       <c r="C66" t="s">
         <v>37</v>
@@ -3235,8 +3237,8 @@
       <c r="A67" s="6">
         <v>45809</v>
       </c>
-      <c r="B67" s="15">
-        <v>349.577</v>
+      <c r="B67" s="42">
+        <v>350.08568656610299</v>
       </c>
       <c r="C67" t="s">
         <v>37</v>
@@ -3252,8 +3254,8 @@
       <c r="A68" s="6">
         <v>45839</v>
       </c>
-      <c r="B68" s="15">
-        <v>348.91199999999998</v>
+      <c r="B68" s="42">
+        <v>350.04962687228198</v>
       </c>
       <c r="C68" t="s">
         <v>37</v>
@@ -3269,8 +3271,8 @@
       <c r="A69" s="6">
         <v>45870</v>
       </c>
-      <c r="B69" s="15">
-        <v>351.822</v>
+      <c r="B69" s="42">
+        <v>352.52850374678297</v>
       </c>
       <c r="C69" t="s">
         <v>37</v>
@@ -3286,8 +3288,8 @@
       <c r="A70" s="6">
         <v>45901</v>
       </c>
-      <c r="B70" s="15">
-        <v>354.90100000000001</v>
+      <c r="B70" s="42">
+        <v>355.21745831006899</v>
       </c>
       <c r="C70" t="s">
         <v>37</v>
@@ -3297,6 +3299,108 @@
       </c>
       <c r="E70" s="6">
         <v>45901</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71" s="6">
+        <v>45931</v>
+      </c>
+      <c r="B71" s="42">
+        <v>359.24574994296302</v>
+      </c>
+      <c r="C71" t="s">
+        <v>37</v>
+      </c>
+      <c r="D71" t="s">
+        <v>23</v>
+      </c>
+      <c r="E71" s="6">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5">
+      <c r="A72" s="6">
+        <v>45962</v>
+      </c>
+      <c r="B72" s="42">
+        <v>360.80766714937101</v>
+      </c>
+      <c r="C72" t="s">
+        <v>37</v>
+      </c>
+      <c r="D72" t="s">
+        <v>23</v>
+      </c>
+      <c r="E72" s="6">
+        <v>45962</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5">
+      <c r="A73" s="6">
+        <v>45992</v>
+      </c>
+      <c r="B73" s="42">
+        <v>361.20040357866702</v>
+      </c>
+      <c r="C73" t="s">
+        <v>37</v>
+      </c>
+      <c r="D73" t="s">
+        <v>23</v>
+      </c>
+      <c r="E73" s="6">
+        <v>45992</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
+      <c r="A74" s="6">
+        <v>46023</v>
+      </c>
+      <c r="B74" s="42">
+        <v>360.98095555893298</v>
+      </c>
+      <c r="C74" t="s">
+        <v>37</v>
+      </c>
+      <c r="D74" t="s">
+        <v>23</v>
+      </c>
+      <c r="E74" s="6">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
+      <c r="A75" s="6">
+        <v>46054</v>
+      </c>
+      <c r="B75" s="42">
+        <v>361.44834672303</v>
+      </c>
+      <c r="C75" t="s">
+        <v>37</v>
+      </c>
+      <c r="D75" t="s">
+        <v>23</v>
+      </c>
+      <c r="E75" s="6">
+        <v>46054</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5">
+      <c r="A76" s="6">
+        <v>46082</v>
+      </c>
+      <c r="B76" s="42">
+        <v>360.15886596558403</v>
+      </c>
+      <c r="C76" t="s">
+        <v>37</v>
+      </c>
+      <c r="D76" t="s">
+        <v>23</v>
+      </c>
+      <c r="E76" s="6">
+        <v>46082</v>
       </c>
     </row>
   </sheetData>
@@ -3308,7 +3412,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F7B815A-330A-FB44-A90A-EA6BA5552924}">
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr defaultColWidth="10.78125" defaultRowHeight="27.5"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -4488,8 +4592,8 @@
       <c r="A70" s="6">
         <v>45901</v>
       </c>
-      <c r="B70" s="10">
-        <v>200.2</v>
+      <c r="B70">
+        <v>199.9</v>
       </c>
       <c r="C70" t="s">
         <v>28</v>
@@ -4505,8 +4609,8 @@
       <c r="A71" s="6">
         <v>45931</v>
       </c>
-      <c r="B71" s="10">
-        <v>200.2</v>
+      <c r="B71">
+        <v>199.9</v>
       </c>
       <c r="C71" t="s">
         <v>28</v>
@@ -4516,6 +4620,108 @@
       </c>
       <c r="E71" s="6">
         <v>45931</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5">
+      <c r="A72" s="6">
+        <v>45962</v>
+      </c>
+      <c r="B72">
+        <v>200.4</v>
+      </c>
+      <c r="C72" t="s">
+        <v>28</v>
+      </c>
+      <c r="D72" t="s">
+        <v>23</v>
+      </c>
+      <c r="E72" s="6">
+        <v>45962</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5">
+      <c r="A73" s="6">
+        <v>45992</v>
+      </c>
+      <c r="B73">
+        <v>200.4</v>
+      </c>
+      <c r="C73" t="s">
+        <v>28</v>
+      </c>
+      <c r="D73" t="s">
+        <v>23</v>
+      </c>
+      <c r="E73" s="6">
+        <v>45992</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
+      <c r="A74" s="6">
+        <v>46023</v>
+      </c>
+      <c r="B74">
+        <v>200.8</v>
+      </c>
+      <c r="C74" t="s">
+        <v>28</v>
+      </c>
+      <c r="D74" t="s">
+        <v>23</v>
+      </c>
+      <c r="E74" s="6">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
+      <c r="A75" s="6">
+        <v>46054</v>
+      </c>
+      <c r="B75">
+        <v>201</v>
+      </c>
+      <c r="C75" t="s">
+        <v>28</v>
+      </c>
+      <c r="D75" t="s">
+        <v>23</v>
+      </c>
+      <c r="E75" s="6">
+        <v>46054</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5">
+      <c r="A76" s="6">
+        <v>46082</v>
+      </c>
+      <c r="B76">
+        <v>202.2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>28</v>
+      </c>
+      <c r="D76" t="s">
+        <v>23</v>
+      </c>
+      <c r="E76" s="6">
+        <v>46082</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5">
+      <c r="A77" s="6">
+        <v>46113</v>
+      </c>
+      <c r="B77">
+        <v>203.4</v>
+      </c>
+      <c r="C77" t="s">
+        <v>28</v>
+      </c>
+      <c r="D77" t="s">
+        <v>23</v>
+      </c>
+      <c r="E77" s="6">
+        <v>46113</v>
       </c>
     </row>
   </sheetData>
@@ -4526,7 +4732,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B5A20CA1-A780-FE4D-9430-35E57D84DFED}">
-  <dimension ref="A1:E70"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr defaultColWidth="10.78125" defaultRowHeight="27.5"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -5717,6 +5923,125 @@
       </c>
       <c r="E70" s="6">
         <v>45901</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71" s="6">
+        <v>45931</v>
+      </c>
+      <c r="B71" s="14">
+        <v>521.37699999999995</v>
+      </c>
+      <c r="C71" t="s">
+        <v>37</v>
+      </c>
+      <c r="D71" t="s">
+        <v>23</v>
+      </c>
+      <c r="E71" s="6">
+        <v>45931</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5">
+      <c r="A72" s="6">
+        <v>45962</v>
+      </c>
+      <c r="B72">
+        <v>522.02599999999995</v>
+      </c>
+      <c r="C72" t="s">
+        <v>37</v>
+      </c>
+      <c r="D72" t="s">
+        <v>23</v>
+      </c>
+      <c r="E72" s="6">
+        <v>45962</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5">
+      <c r="A73" s="6">
+        <v>45992</v>
+      </c>
+      <c r="B73">
+        <v>524.77700000000004</v>
+      </c>
+      <c r="C73" t="s">
+        <v>37</v>
+      </c>
+      <c r="D73" t="s">
+        <v>23</v>
+      </c>
+      <c r="E73" s="6">
+        <v>45992</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
+      <c r="A74" s="6">
+        <v>46023</v>
+      </c>
+      <c r="B74">
+        <v>526.399</v>
+      </c>
+      <c r="C74" t="s">
+        <v>37</v>
+      </c>
+      <c r="D74" t="s">
+        <v>23</v>
+      </c>
+      <c r="E74" s="6">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
+      <c r="A75" s="6">
+        <v>46054</v>
+      </c>
+      <c r="B75">
+        <v>527.20100000000002</v>
+      </c>
+      <c r="C75" t="s">
+        <v>37</v>
+      </c>
+      <c r="D75" t="s">
+        <v>23</v>
+      </c>
+      <c r="E75" s="6">
+        <v>46054</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5">
+      <c r="A76" s="6">
+        <v>46082</v>
+      </c>
+      <c r="B76">
+        <v>528.14700000000005</v>
+      </c>
+      <c r="C76" t="s">
+        <v>37</v>
+      </c>
+      <c r="D76" t="s">
+        <v>23</v>
+      </c>
+      <c r="E76" s="6">
+        <v>46082</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5">
+      <c r="A77" s="6">
+        <v>46113</v>
+      </c>
+      <c r="B77">
+        <v>532.15300000000002</v>
+      </c>
+      <c r="C77" t="s">
+        <v>37</v>
+      </c>
+      <c r="D77" t="s">
+        <v>23</v>
+      </c>
+      <c r="E77" s="6">
+        <v>46113</v>
       </c>
     </row>
   </sheetData>
@@ -5742,14 +6067,14 @@
   <sheetData>
     <row r="1" spans="1:9" ht="27.5" customHeight="1">
       <c r="A1" s="32"/>
-      <c r="B1" s="55" t="s">
+      <c r="B1" s="43" t="s">
         <v>46</v>
       </c>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
       <c r="H1" s="32" t="s">
         <v>47</v>
       </c>
@@ -5785,26 +6110,26 @@
         <v>49</v>
       </c>
       <c r="B3" s="36">
-        <v>91078</v>
+        <v>90930</v>
       </c>
       <c r="C3" s="36">
-        <v>202642</v>
+        <v>229213</v>
       </c>
       <c r="D3" s="36">
-        <v>48523</v>
+        <v>50393</v>
       </c>
       <c r="E3" s="36">
-        <v>61399</v>
+        <v>59090</v>
       </c>
       <c r="F3" s="36">
-        <v>41122</v>
+        <v>42046</v>
       </c>
       <c r="G3" s="35"/>
       <c r="H3" s="35">
-        <v>149679</v>
+        <v>182317</v>
       </c>
       <c r="I3" s="35">
-        <v>1255433</v>
+        <v>1369171</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="27.5" customHeight="1">
@@ -5812,19 +6137,19 @@
         <v>57</v>
       </c>
       <c r="B4" s="36">
-        <v>8853</v>
+        <v>8641</v>
       </c>
       <c r="C4" s="36">
-        <v>35126</v>
+        <v>33800</v>
       </c>
       <c r="D4" s="36">
-        <v>9500</v>
+        <v>9543</v>
       </c>
       <c r="E4" s="36">
-        <v>7593</v>
+        <v>7673</v>
       </c>
       <c r="F4" s="36">
-        <v>12013</v>
+        <v>13033</v>
       </c>
       <c r="G4" s="35"/>
       <c r="H4" s="35"/>
@@ -5859,30 +6184,30 @@
       </c>
       <c r="B6" s="34">
         <f>B4/B5</f>
-        <v>104.15294117647059</v>
+        <v>101.65882352941176</v>
       </c>
       <c r="C6" s="34">
         <f>C4/C5</f>
-        <v>266.10606060606062</v>
+        <v>256.06060606060606</v>
       </c>
       <c r="D6" s="34">
         <f>D4/D5</f>
-        <v>103.26086956521739</v>
+        <v>103.72826086956522</v>
       </c>
       <c r="E6" s="34">
         <f>E4/E5</f>
-        <v>84.36666666666666</v>
+        <v>85.25555555555556</v>
       </c>
       <c r="F6" s="34">
         <f>F4/F5</f>
-        <v>93.124031007751938</v>
+        <v>101.03100775193798</v>
       </c>
       <c r="G6" s="33"/>
       <c r="H6" s="33">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="I6" s="33">
-        <v>3587</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="27.5" customHeight="1">
@@ -5891,35 +6216,35 @@
       </c>
       <c r="B7" s="31">
         <f>B6*12/B3</f>
-        <v>1.3722691474534435E-2</v>
+        <v>1.3415879053700003E-2</v>
       </c>
       <c r="C7" s="31">
         <f>C6*12/C3</f>
-        <v>1.5758197842859464E-2</v>
+        <v>1.3405554103507536E-2</v>
       </c>
       <c r="D7" s="31">
         <f>D6*12/D3</f>
-        <v>2.5536970813482447E-2</v>
+        <v>2.4700635612779204E-2</v>
       </c>
       <c r="E7" s="31">
         <f>E6*12/E3</f>
-        <v>1.6488867896871283E-2</v>
+        <v>1.7313702262086086E-2</v>
       </c>
       <c r="F7" s="31">
         <f>F6*12/F3</f>
-        <v>2.7174951901488824E-2</v>
+        <v>2.8834421657785658E-2</v>
       </c>
       <c r="G7" s="31">
         <f>(SUM(B7:F7))/5</f>
-        <v>1.9736335985847293E-2</v>
+        <v>1.9534038537971699E-2</v>
       </c>
       <c r="H7" s="31">
         <f>H6*12/H3</f>
-        <v>3.3191028801635498E-2</v>
+        <v>2.770997767624522E-2</v>
       </c>
       <c r="I7" s="31">
         <f>I6*12/I3</f>
-        <v>3.4286178553534913E-2</v>
+        <v>3.5057710103412944E-2</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="27.5" customHeight="1">
@@ -5939,7 +6264,7 @@
         <v>3</v>
       </c>
       <c r="F8" s="36">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="27.5" customHeight="1">
@@ -5962,7 +6287,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1808E788-1B69-1D47-87B7-5ECE4822BC1E}">
-  <dimension ref="A1:N73"/>
+  <dimension ref="A1:N79"/>
   <sheetFormatPr defaultColWidth="10.78125" defaultRowHeight="27.5"/>
   <cols>
     <col min="1" max="1" width="10.4765625" bestFit="1" customWidth="1"/>
@@ -8777,32 +9102,242 @@
       </c>
       <c r="B73" s="22">
         <f>rawData_HousePriceIndex_SZ!B73</f>
-        <v>53601</v>
+        <v>53357</v>
       </c>
       <c r="E73" s="8"/>
       <c r="I73" s="16">
-        <f t="shared" ref="I73" si="2">(B73-B72)/B72</f>
-        <v>-2.6050873634655106E-3</v>
+        <f t="shared" ref="I73:I74" si="2">(B73-B72)/B72</f>
+        <v>-7.1453824826482578E-3</v>
       </c>
       <c r="J73" s="16">
         <f>(Processed_CN_SZ[[#This Row],[Value]]-B61)/B61</f>
-        <v>-8.3727926973110656E-2</v>
+        <v>-8.7898938443392194E-2</v>
       </c>
       <c r="K73" s="7">
         <f>Processed_CN_SZ[[#This Row],[Value]]/B72 * 100</f>
-        <v>99.739491263653449</v>
+        <v>99.28546175173517</v>
       </c>
       <c r="L73" s="7">
         <f>Processed_CN_SZ[[#This Row],[Value]]/B61 * 100</f>
-        <v>91.627207302688944</v>
+        <v>91.210106155660782</v>
       </c>
       <c r="M73" cm="1">
         <f t="array" ref="M73">ROUND( Processed_CN_SZ[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_CN_SZ[Value], YEAR(Processed_CN_SZ[Date])=2020) ), 3) * 100</f>
-        <v>96</v>
+        <v>95.5</v>
       </c>
       <c r="N73" s="16" cm="1">
         <f t="array" ref="N73" xml:space="preserve"> Processed_CN_SZ[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_CN_SZ[Date], YEAR(Processed_CN_SZ[Date])=YEAR(Processed_CN_SZ[[#This Row],[Date]]))), Processed_CN_SZ[Date], Processed_CN_SZ[Value]) - 1</f>
-        <v>-8.4025428073413289E-2</v>
+        <v>-8.8195085272907536E-2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14">
+      <c r="A74" s="8">
+        <f>rawData_HousePriceIndex_SZ!A74</f>
+        <v>46023</v>
+      </c>
+      <c r="B74" s="22">
+        <f>rawData_HousePriceIndex_SZ!B74</f>
+        <v>53390</v>
+      </c>
+      <c r="E74" s="8"/>
+      <c r="I74" s="16">
+        <f t="shared" si="2"/>
+        <v>6.1847555147403338E-4</v>
+      </c>
+      <c r="J74" s="16">
+        <f>(Processed_CN_SZ[[#This Row],[Value]]-B62)/B62</f>
+        <v>-8.7631156225434909E-2</v>
+      </c>
+      <c r="K74" s="7">
+        <f>Processed_CN_SZ[[#This Row],[Value]]/B73 * 100</f>
+        <v>100.06184755514739</v>
+      </c>
+      <c r="L74" s="7">
+        <f>Processed_CN_SZ[[#This Row],[Value]]/B62 * 100</f>
+        <v>91.236884377456505</v>
+      </c>
+      <c r="M74" cm="1">
+        <f t="array" ref="M74">ROUND( Processed_CN_SZ[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_CN_SZ[Value], YEAR(Processed_CN_SZ[Date])=2020) ), 3) * 100</f>
+        <v>95.6</v>
+      </c>
+      <c r="N74" s="16" cm="1">
+        <f t="array" ref="N74" xml:space="preserve"> Processed_CN_SZ[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_CN_SZ[Date], YEAR(Processed_CN_SZ[Date])=YEAR(Processed_CN_SZ[[#This Row],[Date]]))), Processed_CN_SZ[Date], Processed_CN_SZ[Value]) - 1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14">
+      <c r="A75" s="8">
+        <f>rawData_HousePriceIndex_SZ!A75</f>
+        <v>46054</v>
+      </c>
+      <c r="B75" s="22">
+        <f>rawData_HousePriceIndex_SZ!B75</f>
+        <v>53781</v>
+      </c>
+      <c r="E75" s="8"/>
+      <c r="I75" s="16">
+        <f t="shared" ref="I75:I78" si="3">(B75-B74)/B74</f>
+        <v>7.3234688143847164E-3</v>
+      </c>
+      <c r="J75" s="16">
+        <f>(Processed_CN_SZ[[#This Row],[Value]]-B63)/B63</f>
+        <v>-9.2227192168115452E-2</v>
+      </c>
+      <c r="K75" s="7">
+        <f>Processed_CN_SZ[[#This Row],[Value]]/B74 * 100</f>
+        <v>100.73234688143846</v>
+      </c>
+      <c r="L75" s="7">
+        <f>Processed_CN_SZ[[#This Row],[Value]]/B63 * 100</f>
+        <v>90.777280783188445</v>
+      </c>
+      <c r="M75" cm="1">
+        <f t="array" ref="M75">ROUND( Processed_CN_SZ[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_CN_SZ[Value], YEAR(Processed_CN_SZ[Date])=2020) ), 3) * 100</f>
+        <v>96.3</v>
+      </c>
+      <c r="N75" s="16" cm="1">
+        <f t="array" ref="N75" xml:space="preserve"> Processed_CN_SZ[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_CN_SZ[Date], YEAR(Processed_CN_SZ[Date])=YEAR(Processed_CN_SZ[[#This Row],[Date]]))), Processed_CN_SZ[Date], Processed_CN_SZ[Value]) - 1</f>
+        <v>7.3234688143846149E-3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14">
+      <c r="A76" s="8">
+        <f>rawData_HousePriceIndex_SZ!A76</f>
+        <v>46082</v>
+      </c>
+      <c r="B76" s="22">
+        <f>rawData_HousePriceIndex_SZ!B76</f>
+        <v>53598</v>
+      </c>
+      <c r="E76" s="8"/>
+      <c r="I76" s="16">
+        <f t="shared" si="3"/>
+        <v>-3.4026886818764993E-3</v>
+      </c>
+      <c r="J76" s="16">
+        <f>(Processed_CN_SZ[[#This Row],[Value]]-B64)/B64</f>
+        <v>-8.513979449015123E-2</v>
+      </c>
+      <c r="K76" s="7">
+        <f>Processed_CN_SZ[[#This Row],[Value]]/B75 * 100</f>
+        <v>99.65973113181235</v>
+      </c>
+      <c r="L76" s="7">
+        <f>Processed_CN_SZ[[#This Row],[Value]]/B64 * 100</f>
+        <v>91.486020550984875</v>
+      </c>
+      <c r="M76" cm="1">
+        <f t="array" ref="M76">ROUND( Processed_CN_SZ[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_CN_SZ[Value], YEAR(Processed_CN_SZ[Date])=2020) ), 3) * 100</f>
+        <v>96</v>
+      </c>
+      <c r="N76" s="16" cm="1">
+        <f t="array" ref="N76" xml:space="preserve"> Processed_CN_SZ[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_CN_SZ[Date], YEAR(Processed_CN_SZ[Date])=YEAR(Processed_CN_SZ[[#This Row],[Date]]))), Processed_CN_SZ[Date], Processed_CN_SZ[Value]) - 1</f>
+        <v>3.8958606480614666E-3</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14">
+      <c r="A77" s="8">
+        <f>rawData_HousePriceIndex_SZ!A77</f>
+        <v>46113</v>
+      </c>
+      <c r="B77" s="22">
+        <f>rawData_HousePriceIndex_SZ!B77</f>
+        <v>53066</v>
+      </c>
+      <c r="E77" s="8"/>
+      <c r="I77" s="16">
+        <f t="shared" si="3"/>
+        <v>-9.925743497891713E-3</v>
+      </c>
+      <c r="J77" s="16">
+        <f>(Processed_CN_SZ[[#This Row],[Value]]-B65)/B65</f>
+        <v>-8.2791758849557529E-2</v>
+      </c>
+      <c r="K77" s="7">
+        <f>Processed_CN_SZ[[#This Row],[Value]]/B76 * 100</f>
+        <v>99.007425650210834</v>
+      </c>
+      <c r="L77" s="7">
+        <f>Processed_CN_SZ[[#This Row],[Value]]/B65 * 100</f>
+        <v>91.720824115044252</v>
+      </c>
+      <c r="M77" cm="1">
+        <f t="array" ref="M77">ROUND( Processed_CN_SZ[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_CN_SZ[Value], YEAR(Processed_CN_SZ[Date])=2020) ), 3) * 100</f>
+        <v>95</v>
+      </c>
+      <c r="N77" s="16" cm="1">
+        <f t="array" ref="N77" xml:space="preserve"> Processed_CN_SZ[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_CN_SZ[Date], YEAR(Processed_CN_SZ[Date])=YEAR(Processed_CN_SZ[[#This Row],[Date]]))), Processed_CN_SZ[Date], Processed_CN_SZ[Value]) - 1</f>
+        <v>-6.0685521633264683E-3</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14">
+      <c r="A78" s="8">
+        <f>rawData_HousePriceIndex_SZ!A78</f>
+        <v>46143</v>
+      </c>
+      <c r="B78" s="22">
+        <f>rawData_HousePriceIndex_SZ!B78</f>
+        <v>52386</v>
+      </c>
+      <c r="E78" s="8"/>
+      <c r="I78" s="16">
+        <f t="shared" si="3"/>
+        <v>-1.2814231334564505E-2</v>
+      </c>
+      <c r="J78" s="16">
+        <f>(Processed_CN_SZ[[#This Row],[Value]]-B66)/B66</f>
+        <v>-9.4028327828026906E-2</v>
+      </c>
+      <c r="K78" s="7">
+        <f>Processed_CN_SZ[[#This Row],[Value]]/B77 * 100</f>
+        <v>98.718576866543543</v>
+      </c>
+      <c r="L78" s="7">
+        <f>Processed_CN_SZ[[#This Row],[Value]]/B66 * 100</f>
+        <v>90.59716721719731</v>
+      </c>
+      <c r="M78" cm="1">
+        <f t="array" ref="M78">ROUND( Processed_CN_SZ[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_CN_SZ[Value], YEAR(Processed_CN_SZ[Date])=2020) ), 3) * 100</f>
+        <v>93.8</v>
+      </c>
+      <c r="N78" s="16" cm="1">
+        <f t="array" ref="N78" xml:space="preserve"> Processed_CN_SZ[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_CN_SZ[Date], YEAR(Processed_CN_SZ[Date])=YEAR(Processed_CN_SZ[[#This Row],[Date]]))), Processed_CN_SZ[Date], Processed_CN_SZ[Value]) - 1</f>
+        <v>-1.8805019666604195E-2</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14">
+      <c r="A79" s="8">
+        <f>rawData_HousePriceIndex_SZ!A79</f>
+        <v>46174</v>
+      </c>
+      <c r="B79" s="22">
+        <f>rawData_HousePriceIndex_SZ!B79</f>
+        <v>52253</v>
+      </c>
+      <c r="E79" s="8"/>
+      <c r="I79" s="16">
+        <f t="shared" ref="I79" si="4">(B79-B78)/B78</f>
+        <v>-2.5388462566334519E-3</v>
+      </c>
+      <c r="J79" s="16">
+        <f>(Processed_CN_SZ[[#This Row],[Value]]-B67)/B67</f>
+        <v>-8.2636938202247184E-2</v>
+      </c>
+      <c r="K79" s="7">
+        <f>Processed_CN_SZ[[#This Row],[Value]]/B78 * 100</f>
+        <v>99.746115374336654</v>
+      </c>
+      <c r="L79" s="7">
+        <f>Processed_CN_SZ[[#This Row],[Value]]/B67 * 100</f>
+        <v>91.736306179775283</v>
+      </c>
+      <c r="M79" cm="1">
+        <f t="array" ref="M79">ROUND( Processed_CN_SZ[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_CN_SZ[Value], YEAR(Processed_CN_SZ[Date])=2020) ), 3) * 100</f>
+        <v>93.600000000000009</v>
+      </c>
+      <c r="N79" s="16" cm="1">
+        <f t="array" ref="N79" xml:space="preserve"> Processed_CN_SZ[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_CN_SZ[Date], YEAR(Processed_CN_SZ[Date])=YEAR(Processed_CN_SZ[[#This Row],[Date]]))), Processed_CN_SZ[Date], Processed_CN_SZ[Value]) - 1</f>
+        <v>-2.1296122869451262E-2</v>
       </c>
     </row>
   </sheetData>
@@ -8817,7 +9352,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6FF786FB-40B9-A444-B135-8903222623C0}">
-  <dimension ref="A1:N71"/>
+  <dimension ref="A1:N77"/>
   <sheetFormatPr defaultColWidth="10.78125" defaultRowHeight="27.5"/>
   <cols>
     <col min="1" max="1" width="9.4765625" bestFit="1" customWidth="1"/>
@@ -12280,7 +12815,7 @@
       </c>
       <c r="B70" s="10">
         <f>rawData_HousePriceIndex_HK!B70</f>
-        <v>293.10000000000002</v>
+        <v>293.39999999999998</v>
       </c>
       <c r="C70" t="s">
         <v>35</v>
@@ -12288,27 +12823,27 @@
       <c r="E70" s="8"/>
       <c r="I70" s="16">
         <f t="shared" si="1"/>
-        <v>1.5240734326290386E-2</v>
+        <v>1.6279875303082746E-2</v>
       </c>
       <c r="J70" s="16">
         <f>(Processed_CN_HK[[#This Row],[Value]]-B58)/B58</f>
-        <v>1.806182702327213E-2</v>
+        <v>1.9103855505383814E-2</v>
       </c>
       <c r="K70" s="7">
         <f>Processed_CN_HK[[#This Row],[Value]]/B69 * 100</f>
-        <v>101.52407343262904</v>
+        <v>101.62798753030829</v>
       </c>
       <c r="L70" s="7">
         <f>Processed_CN_HK[[#This Row],[Value]]/B58 * 100</f>
-        <v>101.80618270232722</v>
+        <v>101.91038555053838</v>
       </c>
       <c r="M70" cm="1">
         <f t="array" ref="M70">ROUND( Processed_CN_HK[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_CN_HK[Value], YEAR(Processed_CN_HK[Date])=2020) ), 3) * 100</f>
-        <v>76.900000000000006</v>
+        <v>77</v>
       </c>
       <c r="N70" s="16" cm="1">
         <f t="array" ref="N70" xml:space="preserve"> Processed_CN_HK[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_CN_HK[Date], YEAR(Processed_CN_HK[Date])=YEAR(Processed_CN_HK[[#This Row],[Date]]))), Processed_CN_HK[Date], Processed_CN_HK[Value]) - 1</f>
-        <v>2.0543175487465204E-2</v>
+        <v>2.1587743732590425E-2</v>
       </c>
     </row>
     <row r="71" spans="1:14">
@@ -12318,7 +12853,7 @@
       </c>
       <c r="B71" s="10">
         <f>rawData_HousePriceIndex_HK!B71</f>
-        <v>294.3</v>
+        <v>294.89999999999998</v>
       </c>
       <c r="C71" t="s">
         <v>35</v>
@@ -12340,27 +12875,297 @@
       </c>
       <c r="I71" s="16">
         <f t="shared" ref="I71:I72" si="2">(B71-B70)/B70</f>
-        <v>4.0941658137154165E-3</v>
+        <v>5.1124744376278121E-3</v>
       </c>
       <c r="J71" s="16">
         <f>(Processed_CN_HK[[#This Row],[Value]]-B59)/B59</f>
-        <v>1.134020618556705E-2</v>
+        <v>1.3402061855670024E-2</v>
       </c>
       <c r="K71" s="7">
         <f>Processed_CN_HK[[#This Row],[Value]]/B70 * 100</f>
-        <v>100.40941658137154</v>
+        <v>100.51124744376278</v>
       </c>
       <c r="L71" s="7">
         <f>Processed_CN_HK[[#This Row],[Value]]/B59 * 100</f>
-        <v>101.13402061855669</v>
+        <v>101.34020618556701</v>
       </c>
       <c r="M71" cm="1">
         <f t="array" ref="M71">ROUND( Processed_CN_HK[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_CN_HK[Value], YEAR(Processed_CN_HK[Date])=2020) ), 3) * 100</f>
-        <v>77.2</v>
+        <v>77.400000000000006</v>
       </c>
       <c r="N71" s="16" cm="1">
         <f t="array" ref="N71" xml:space="preserve"> Processed_CN_HK[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_CN_HK[Date], YEAR(Processed_CN_HK[Date])=YEAR(Processed_CN_HK[[#This Row],[Date]]))), Processed_CN_HK[Date], Processed_CN_HK[Value]) - 1</f>
-        <v>2.4721448467966756E-2</v>
+        <v>2.6810584958217198E-2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14">
+      <c r="A72" s="6">
+        <f>rawData_HousePriceIndex_HK!A72</f>
+        <v>45962</v>
+      </c>
+      <c r="B72" s="10">
+        <f>rawData_HousePriceIndex_HK!B72</f>
+        <v>298.7</v>
+      </c>
+      <c r="C72" t="s">
+        <v>35</v>
+      </c>
+      <c r="E72" s="8"/>
+      <c r="I72" s="16">
+        <f t="shared" si="2"/>
+        <v>1.2885723974228592E-2</v>
+      </c>
+      <c r="J72" s="16">
+        <f>(Processed_CN_HK[[#This Row],[Value]]-B60)/B60</f>
+        <v>2.469982847341334E-2</v>
+      </c>
+      <c r="K72" s="7">
+        <f>Processed_CN_HK[[#This Row],[Value]]/B71 * 100</f>
+        <v>101.28857239742285</v>
+      </c>
+      <c r="L72" s="7">
+        <f>Processed_CN_HK[[#This Row],[Value]]/B60 * 100</f>
+        <v>102.46998284734133</v>
+      </c>
+      <c r="M72" cm="1">
+        <f t="array" ref="M72">ROUND( Processed_CN_HK[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_CN_HK[Value], YEAR(Processed_CN_HK[Date])=2020) ), 3) * 100</f>
+        <v>78.400000000000006</v>
+      </c>
+      <c r="N72" s="16" cm="1">
+        <f t="array" ref="N72" xml:space="preserve"> Processed_CN_HK[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_CN_HK[Date], YEAR(Processed_CN_HK[Date])=YEAR(Processed_CN_HK[[#This Row],[Date]]))), Processed_CN_HK[Date], Processed_CN_HK[Value]) - 1</f>
+        <v>4.0041782729804964E-2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14">
+      <c r="A73" s="6">
+        <f>rawData_HousePriceIndex_HK!A73</f>
+        <v>45992</v>
+      </c>
+      <c r="B73" s="10">
+        <f>rawData_HousePriceIndex_HK!B73</f>
+        <v>299.60000000000002</v>
+      </c>
+      <c r="C73" t="s">
+        <v>35</v>
+      </c>
+      <c r="D73" t="s">
+        <v>22</v>
+      </c>
+      <c r="E73" s="8">
+        <v>45872</v>
+      </c>
+      <c r="F73">
+        <v>67</v>
+      </c>
+      <c r="G73">
+        <v>288</v>
+      </c>
+      <c r="H73">
+        <v>292</v>
+      </c>
+      <c r="I73" s="16">
+        <f t="shared" ref="I73:I76" si="3">(B73-B72)/B72</f>
+        <v>3.0130565785069772E-3</v>
+      </c>
+      <c r="J73" s="16">
+        <f>(Processed_CN_HK[[#This Row],[Value]]-B61)/B61</f>
+        <v>3.5961272475795419E-2</v>
+      </c>
+      <c r="K73" s="7">
+        <f>Processed_CN_HK[[#This Row],[Value]]/B72 * 100</f>
+        <v>100.30130565785069</v>
+      </c>
+      <c r="L73" s="7">
+        <f>Processed_CN_HK[[#This Row],[Value]]/B61 * 100</f>
+        <v>103.59612724757955</v>
+      </c>
+      <c r="M73" cm="1">
+        <f t="array" ref="M73">ROUND( Processed_CN_HK[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_CN_HK[Value], YEAR(Processed_CN_HK[Date])=2020) ), 3) * 100</f>
+        <v>78.600000000000009</v>
+      </c>
+      <c r="N73" s="16" cm="1">
+        <f t="array" ref="N73" xml:space="preserve"> Processed_CN_HK[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_CN_HK[Date], YEAR(Processed_CN_HK[Date])=YEAR(Processed_CN_HK[[#This Row],[Date]]))), Processed_CN_HK[Date], Processed_CN_HK[Value]) - 1</f>
+        <v>4.3175487465181073E-2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14">
+      <c r="A74" s="6">
+        <f>rawData_HousePriceIndex_HK!A74</f>
+        <v>46023</v>
+      </c>
+      <c r="B74" s="10">
+        <f>rawData_HousePriceIndex_HK!B74</f>
+        <v>303</v>
+      </c>
+      <c r="C74" t="s">
+        <v>35</v>
+      </c>
+      <c r="E74" s="8"/>
+      <c r="I74" s="16">
+        <f t="shared" si="3"/>
+        <v>1.134846461949258E-2</v>
+      </c>
+      <c r="J74" s="16">
+        <f>(Processed_CN_HK[[#This Row],[Value]]-B62)/B62</f>
+        <v>5.5013927576601715E-2</v>
+      </c>
+      <c r="K74" s="7">
+        <f>Processed_CN_HK[[#This Row],[Value]]/B73 * 100</f>
+        <v>101.13484646194925</v>
+      </c>
+      <c r="L74" s="7">
+        <f>Processed_CN_HK[[#This Row],[Value]]/B62 * 100</f>
+        <v>105.50139275766017</v>
+      </c>
+      <c r="M74" cm="1">
+        <f t="array" ref="M74">ROUND( Processed_CN_HK[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_CN_HK[Value], YEAR(Processed_CN_HK[Date])=2020) ), 3) * 100</f>
+        <v>79.5</v>
+      </c>
+      <c r="N74" s="16" cm="1">
+        <f t="array" ref="N74" xml:space="preserve"> Processed_CN_HK[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_CN_HK[Date], YEAR(Processed_CN_HK[Date])=YEAR(Processed_CN_HK[[#This Row],[Date]]))), Processed_CN_HK[Date], Processed_CN_HK[Value]) - 1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14">
+      <c r="A75" s="6">
+        <f>rawData_HousePriceIndex_HK!A75</f>
+        <v>46054</v>
+      </c>
+      <c r="B75" s="10">
+        <f>rawData_HousePriceIndex_HK!B75</f>
+        <v>308.5</v>
+      </c>
+      <c r="C75" t="s">
+        <v>35</v>
+      </c>
+      <c r="D75" t="s">
+        <v>22</v>
+      </c>
+      <c r="E75" s="8">
+        <v>45873</v>
+      </c>
+      <c r="F75">
+        <v>67</v>
+      </c>
+      <c r="G75">
+        <v>288</v>
+      </c>
+      <c r="H75">
+        <v>292</v>
+      </c>
+      <c r="I75" s="16">
+        <f t="shared" si="3"/>
+        <v>1.8151815181518153E-2</v>
+      </c>
+      <c r="J75" s="16">
+        <f>(Processed_CN_HK[[#This Row],[Value]]-B63)/B63</f>
+        <v>8.0182072829131562E-2</v>
+      </c>
+      <c r="K75" s="7">
+        <f>Processed_CN_HK[[#This Row],[Value]]/B74 * 100</f>
+        <v>101.8151815181518</v>
+      </c>
+      <c r="L75" s="7">
+        <f>Processed_CN_HK[[#This Row],[Value]]/B63 * 100</f>
+        <v>108.01820728291315</v>
+      </c>
+      <c r="M75" cm="1">
+        <f t="array" ref="M75">ROUND( Processed_CN_HK[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_CN_HK[Value], YEAR(Processed_CN_HK[Date])=2020) ), 3) * 100</f>
+        <v>80.900000000000006</v>
+      </c>
+      <c r="N75" s="16" cm="1">
+        <f t="array" ref="N75" xml:space="preserve"> Processed_CN_HK[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_CN_HK[Date], YEAR(Processed_CN_HK[Date])=YEAR(Processed_CN_HK[[#This Row],[Date]]))), Processed_CN_HK[Date], Processed_CN_HK[Value]) - 1</f>
+        <v>1.8151815181518094E-2</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14">
+      <c r="A76" s="6">
+        <f>rawData_HousePriceIndex_HK!A76</f>
+        <v>46082</v>
+      </c>
+      <c r="B76" s="10">
+        <f>rawData_HousePriceIndex_HK!B76</f>
+        <v>312.8</v>
+      </c>
+      <c r="C76" t="s">
+        <v>35</v>
+      </c>
+      <c r="E76" s="8"/>
+      <c r="I76" s="16">
+        <f t="shared" si="3"/>
+        <v>1.3938411669367946E-2</v>
+      </c>
+      <c r="J76" s="16">
+        <f>(Processed_CN_HK[[#This Row],[Value]]-B64)/B64</f>
+        <v>9.7929097929098055E-2</v>
+      </c>
+      <c r="K76" s="7">
+        <f>Processed_CN_HK[[#This Row],[Value]]/B75 * 100</f>
+        <v>101.3938411669368</v>
+      </c>
+      <c r="L76" s="7">
+        <f>Processed_CN_HK[[#This Row],[Value]]/B64 * 100</f>
+        <v>109.79290979290981</v>
+      </c>
+      <c r="M76" cm="1">
+        <f t="array" ref="M76">ROUND( Processed_CN_HK[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_CN_HK[Value], YEAR(Processed_CN_HK[Date])=2020) ), 3) * 100</f>
+        <v>82.1</v>
+      </c>
+      <c r="N76" s="16" cm="1">
+        <f t="array" ref="N76" xml:space="preserve"> Processed_CN_HK[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_CN_HK[Date], YEAR(Processed_CN_HK[Date])=YEAR(Processed_CN_HK[[#This Row],[Date]]))), Processed_CN_HK[Date], Processed_CN_HK[Value]) - 1</f>
+        <v>3.2343234323432446E-2</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14">
+      <c r="A77" s="6">
+        <f>rawData_HousePriceIndex_HK!A77</f>
+        <v>46113</v>
+      </c>
+      <c r="B77" s="10">
+        <f>rawData_HousePriceIndex_HK!B77</f>
+        <v>316.60000000000002</v>
+      </c>
+      <c r="C77" t="s">
+        <v>35</v>
+      </c>
+      <c r="D77" t="s">
+        <v>22</v>
+      </c>
+      <c r="E77" s="8">
+        <v>45874</v>
+      </c>
+      <c r="F77">
+        <v>67</v>
+      </c>
+      <c r="G77">
+        <v>288</v>
+      </c>
+      <c r="H77">
+        <v>292</v>
+      </c>
+      <c r="I77" s="16">
+        <f t="shared" ref="I77" si="4">(B77-B76)/B76</f>
+        <v>1.2148337595907964E-2</v>
+      </c>
+      <c r="J77" s="16">
+        <f>(Processed_CN_HK[[#This Row],[Value]]-B65)/B65</f>
+        <v>0.10506108202443289</v>
+      </c>
+      <c r="K77" s="7">
+        <f>Processed_CN_HK[[#This Row],[Value]]/B76 * 100</f>
+        <v>101.21483375959079</v>
+      </c>
+      <c r="L77" s="7">
+        <f>Processed_CN_HK[[#This Row],[Value]]/B65 * 100</f>
+        <v>110.50610820244329</v>
+      </c>
+      <c r="M77" cm="1">
+        <f t="array" ref="M77">ROUND( Processed_CN_HK[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_CN_HK[Value], YEAR(Processed_CN_HK[Date])=2020) ), 3) * 100</f>
+        <v>83.1</v>
+      </c>
+      <c r="N77" s="16" cm="1">
+        <f t="array" ref="N77" xml:space="preserve"> Processed_CN_HK[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_CN_HK[Date], YEAR(Processed_CN_HK[Date])=YEAR(Processed_CN_HK[[#This Row],[Date]]))), Processed_CN_HK[Date], Processed_CN_HK[Value]) - 1</f>
+        <v>4.488448844884485E-2</v>
       </c>
     </row>
   </sheetData>
@@ -12375,7 +13180,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03EFFF24-D6EE-8F4D-AB5E-F4F62FCFEC7D}">
-  <dimension ref="A1:N70"/>
+  <dimension ref="A1:N76"/>
   <sheetFormatPr defaultColWidth="10.78125" defaultRowHeight="27.5"/>
   <cols>
     <col min="1" max="1" width="9.4765625" bestFit="1" customWidth="1"/>
@@ -15591,7 +16396,7 @@
       </c>
       <c r="B65" s="21">
         <f>rawData_HousePriceIndex_US!B65</f>
-        <v>354.17</v>
+        <v>354.19372711900598</v>
       </c>
       <c r="C65" t="s">
         <v>36</v>
@@ -15613,27 +16418,27 @@
       </c>
       <c r="I65" s="16">
         <f t="shared" si="0"/>
-        <v>-1.1987156418861342E-2</v>
+        <v>-1.1920965893635956E-2</v>
       </c>
       <c r="J65" s="16">
         <f>(Processed_US_CA[[#This Row],[Value]]-B53)/B53</f>
-        <v>1.4137472785364887E-3</v>
+        <v>1.4808355783808881E-3</v>
       </c>
       <c r="K65" s="7">
         <f>Processed_US_CA[[#This Row],[Value]]/B64 * 100</f>
-        <v>98.801284358113861</v>
+        <v>98.807903410636399</v>
       </c>
       <c r="L65" s="7">
         <f>Processed_US_CA[[#This Row],[Value]]/B53 * 100</f>
-        <v>100.14137472785364</v>
+        <v>100.14808355783809</v>
       </c>
       <c r="M65" cm="1">
         <f t="array" ref="M65">ROUND( Processed_US_CA[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_US_CA[Value], YEAR(Processed_US_CA[Date])=2020) ), 3) * 100</f>
-        <v>126.89999999999999</v>
+        <v>127</v>
       </c>
       <c r="N65" s="16" cm="1">
         <f t="array" ref="N65" xml:space="preserve"> Processed_US_CA[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_US_CA[Date], YEAR(Processed_US_CA[Date])=YEAR(Processed_US_CA[[#This Row],[Date]]))), Processed_US_CA[Date], Processed_US_CA[Value]) - 1</f>
-        <v>-2.4556165756873027E-2</v>
+        <v>-2.4490817274678833E-2</v>
       </c>
     </row>
     <row r="66" spans="1:14">
@@ -15643,7 +16448,7 @@
       </c>
       <c r="B66" s="21">
         <f>rawData_HousePriceIndex_US!B66</f>
-        <v>351.71199999999999</v>
+        <v>352.11270457490201</v>
       </c>
       <c r="C66" t="s">
         <v>36</v>
@@ -15665,27 +16470,27 @@
       </c>
       <c r="I66" s="16">
         <f t="shared" si="0"/>
-        <v>-6.9401699748709005E-3</v>
+        <v>-5.8753794456804934E-3</v>
       </c>
       <c r="J66" s="16">
         <f>(Processed_US_CA[[#This Row],[Value]]-B54)/B54</f>
-        <v>-7.4362136549765935E-3</v>
+        <v>-6.3053882919792432E-3</v>
       </c>
       <c r="K66" s="7">
         <f>Processed_US_CA[[#This Row],[Value]]/B65 * 100</f>
-        <v>99.305983002512903</v>
+        <v>99.412462055431945</v>
       </c>
       <c r="L66" s="7">
         <f>Processed_US_CA[[#This Row],[Value]]/B54 * 100</f>
-        <v>99.25637863450234</v>
+        <v>99.369461170802083</v>
       </c>
       <c r="M66" cm="1">
         <f t="array" ref="M66">ROUND( Processed_US_CA[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_US_CA[Value], YEAR(Processed_US_CA[Date])=2020) ), 3) * 100</f>
-        <v>126.1</v>
+        <v>126.2</v>
       </c>
       <c r="N66" s="16" cm="1">
         <f t="array" ref="N66" xml:space="preserve"> Processed_US_CA[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_US_CA[Date], YEAR(Processed_US_CA[Date])=YEAR(Processed_US_CA[[#This Row],[Date]]))), Processed_US_CA[Date], Processed_US_CA[Value]) - 1</f>
-        <v>-3.1325911767460135E-2</v>
+        <v>-3.0222303875935719E-2</v>
       </c>
     </row>
     <row r="67" spans="1:14">
@@ -15695,7 +16500,7 @@
       </c>
       <c r="B67" s="21">
         <f>rawData_HousePriceIndex_US!B67</f>
-        <v>349.577</v>
+        <v>350.08568656610299</v>
       </c>
       <c r="C67" t="s">
         <v>36</v>
@@ -15717,27 +16522,27 @@
       </c>
       <c r="I67" s="16">
         <f t="shared" si="0"/>
-        <v>-6.0703075243380691E-3</v>
+        <v>-5.7567306787359267E-3</v>
       </c>
       <c r="J67" s="16">
         <f>(Processed_US_CA[[#This Row],[Value]]-B55)/B55</f>
-        <v>-2.0416798603385616E-2</v>
+        <v>-1.8991359244015227E-2</v>
       </c>
       <c r="K67" s="7">
         <f>Processed_US_CA[[#This Row],[Value]]/B66 * 100</f>
-        <v>99.392969247566199</v>
+        <v>99.424326932126405</v>
       </c>
       <c r="L67" s="7">
         <f>Processed_US_CA[[#This Row],[Value]]/B55 * 100</f>
-        <v>97.958320139661438</v>
+        <v>98.10086407559848</v>
       </c>
       <c r="M67" cm="1">
         <f t="array" ref="M67">ROUND( Processed_US_CA[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_US_CA[Value], YEAR(Processed_US_CA[Date])=2020) ), 3) * 100</f>
-        <v>125.29999999999998</v>
+        <v>125.49999999999999</v>
       </c>
       <c r="N67" s="16" cm="1">
         <f t="array" ref="N67" xml:space="preserve"> Processed_US_CA[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_US_CA[Date], YEAR(Processed_US_CA[Date])=YEAR(Processed_US_CA[[#This Row],[Date]]))), Processed_US_CA[Date], Processed_US_CA[Value]) - 1</f>
-        <v>-3.7206061373889376E-2</v>
+        <v>-3.5805052890766964E-2</v>
       </c>
     </row>
     <row r="68" spans="1:14">
@@ -15747,7 +16552,7 @@
       </c>
       <c r="B68" s="21">
         <f>rawData_HousePriceIndex_US!B68</f>
-        <v>348.91199999999998</v>
+        <v>350.04962687228198</v>
       </c>
       <c r="C68" t="s">
         <v>36</v>
@@ -15769,27 +16574,27 @@
       </c>
       <c r="I68" s="16">
         <f t="shared" ref="I68:I69" si="1">(B68-B67)/B67</f>
-        <v>-1.9022990642977669E-3</v>
+        <v>-1.0300247969209021E-4</v>
       </c>
       <c r="J68" s="16">
         <f>(Processed_US_CA[[#This Row],[Value]]-B56)/B56</f>
-        <v>-1.9673291862641003E-2</v>
+        <v>-1.6476938607972745E-2</v>
       </c>
       <c r="K68" s="7">
         <f>Processed_US_CA[[#This Row],[Value]]/B67 * 100</f>
-        <v>99.809770093570222</v>
+        <v>99.989699752030788</v>
       </c>
       <c r="L68" s="7">
         <f>Processed_US_CA[[#This Row],[Value]]/B56 * 100</f>
-        <v>98.032670813735905</v>
+        <v>98.352306139202724</v>
       </c>
       <c r="M68" cm="1">
         <f t="array" ref="M68">ROUND( Processed_US_CA[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_US_CA[Value], YEAR(Processed_US_CA[Date])=2020) ), 3) * 100</f>
-        <v>125.1</v>
+        <v>125.49999999999999</v>
       </c>
       <c r="N68" s="16" cm="1">
         <f t="array" ref="N68" xml:space="preserve"> Processed_US_CA[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_US_CA[Date], YEAR(Processed_US_CA[Date])=YEAR(Processed_US_CA[[#This Row],[Date]]))), Processed_US_CA[Date], Processed_US_CA[Value]) - 1</f>
-        <v>-3.9037583382449448E-2</v>
+        <v>-3.590436736122582E-2</v>
       </c>
     </row>
     <row r="69" spans="1:14">
@@ -15799,7 +16604,7 @@
       </c>
       <c r="B69" s="21">
         <f>rawData_HousePriceIndex_US!B69</f>
-        <v>351.822</v>
+        <v>352.52850374678297</v>
       </c>
       <c r="C69" t="s">
         <v>36</v>
@@ -15807,27 +16612,27 @@
       <c r="E69" s="8"/>
       <c r="I69" s="16">
         <f t="shared" si="1"/>
-        <v>8.3402118585775929E-3</v>
+        <v>7.0815012621208498E-3</v>
       </c>
       <c r="J69" s="16">
         <f>(Processed_US_CA[[#This Row],[Value]]-B57)/B57</f>
-        <v>-1.5113893080194056E-2</v>
+        <v>-1.3136115326974141E-2</v>
       </c>
       <c r="K69" s="7">
         <f>Processed_US_CA[[#This Row],[Value]]/B68 * 100</f>
-        <v>100.83402118585776</v>
+        <v>100.70815012621208</v>
       </c>
       <c r="L69" s="7">
         <f>Processed_US_CA[[#This Row],[Value]]/B57 * 100</f>
-        <v>98.488610691980597</v>
+        <v>98.686388467302592</v>
       </c>
       <c r="M69" cm="1">
         <f t="array" ref="M69">ROUND( Processed_US_CA[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_US_CA[Value], YEAR(Processed_US_CA[Date])=2020) ), 3) * 100</f>
-        <v>126.1</v>
+        <v>126.4</v>
       </c>
       <c r="N69" s="16" cm="1">
         <f t="array" ref="N69" xml:space="preserve"> Processed_US_CA[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_US_CA[Date], YEAR(Processed_US_CA[Date])=YEAR(Processed_US_CA[[#This Row],[Date]]))), Processed_US_CA[Date], Processed_US_CA[Value]) - 1</f>
-        <v>-3.1022953239728368E-2</v>
+        <v>-2.9077122921889131E-2</v>
       </c>
     </row>
     <row r="70" spans="1:14">
@@ -15837,7 +16642,7 @@
       </c>
       <c r="B70" s="21">
         <f>rawData_HousePriceIndex_US!B70</f>
-        <v>354.90100000000001</v>
+        <v>355.21745831006899</v>
       </c>
       <c r="C70" t="s">
         <v>36</v>
@@ -15858,28 +16663,298 @@
         <v>326</v>
       </c>
       <c r="I70" s="16">
-        <f t="shared" ref="I70" si="2">(B70-B69)/B69</f>
-        <v>8.7515846081257214E-3</v>
+        <f t="shared" ref="I70:I71" si="2">(B70-B69)/B69</f>
+        <v>7.6276231133283389E-3</v>
       </c>
       <c r="J70" s="16">
         <f>(Processed_US_CA[[#This Row],[Value]]-B58)/B58</f>
-        <v>-9.2403639195892985E-3</v>
+        <v>-8.3569228469561833E-3</v>
       </c>
       <c r="K70" s="7">
         <f>Processed_US_CA[[#This Row],[Value]]/B69 * 100</f>
-        <v>100.87515846081257</v>
+        <v>100.76276231133284</v>
       </c>
       <c r="L70" s="7">
         <f>Processed_US_CA[[#This Row],[Value]]/B58 * 100</f>
-        <v>99.075963608041079</v>
+        <v>99.164307715304375</v>
       </c>
       <c r="M70" cm="1">
         <f t="array" ref="M70">ROUND( Processed_US_CA[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_US_CA[Value], YEAR(Processed_US_CA[Date])=2020) ), 3) * 100</f>
-        <v>127.2</v>
+        <v>127.3</v>
       </c>
       <c r="N70" s="16" cm="1">
         <f t="array" ref="N70" xml:space="preserve"> Processed_US_CA[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_US_CA[Date], YEAR(Processed_US_CA[Date])=YEAR(Processed_US_CA[[#This Row],[Date]]))), Processed_US_CA[Date], Processed_US_CA[Value]) - 1</f>
-        <v>-2.2542868631674096E-2</v>
+        <v>-2.1671289143428862E-2</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14">
+      <c r="A71" s="6">
+        <f>rawData_HousePriceIndex_US!A71</f>
+        <v>45931</v>
+      </c>
+      <c r="B71" s="21">
+        <f>rawData_HousePriceIndex_US!B71</f>
+        <v>359.24574994296302</v>
+      </c>
+      <c r="C71" t="s">
+        <v>36</v>
+      </c>
+      <c r="E71" s="8"/>
+      <c r="I71" s="16">
+        <f t="shared" si="2"/>
+        <v>1.1340353742911286E-2</v>
+      </c>
+      <c r="J71" s="16">
+        <f>(Processed_US_CA[[#This Row],[Value]]-B59)/B59</f>
+        <v>4.9224506421606789E-4</v>
+      </c>
+      <c r="K71" s="7">
+        <f>Processed_US_CA[[#This Row],[Value]]/B70 * 100</f>
+        <v>101.13403537429113</v>
+      </c>
+      <c r="L71" s="7">
+        <f>Processed_US_CA[[#This Row],[Value]]/B59 * 100</f>
+        <v>100.0492245064216</v>
+      </c>
+      <c r="M71" cm="1">
+        <f t="array" ref="M71">ROUND( Processed_US_CA[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_US_CA[Value], YEAR(Processed_US_CA[Date])=2020) ), 3) * 100</f>
+        <v>128.80000000000001</v>
+      </c>
+      <c r="N71" s="16" cm="1">
+        <f t="array" ref="N71" xml:space="preserve"> Processed_US_CA[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_US_CA[Date], YEAR(Processed_US_CA[Date])=YEAR(Processed_US_CA[[#This Row],[Date]]))), Processed_US_CA[Date], Processed_US_CA[Value]) - 1</f>
+        <v>-1.0576695485469023E-2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14">
+      <c r="A72" s="6">
+        <f>rawData_HousePriceIndex_US!A72</f>
+        <v>45962</v>
+      </c>
+      <c r="B72" s="21">
+        <f>rawData_HousePriceIndex_US!B72</f>
+        <v>360.80766714937101</v>
+      </c>
+      <c r="C72" t="s">
+        <v>36</v>
+      </c>
+      <c r="D72" t="s">
+        <v>22</v>
+      </c>
+      <c r="E72" s="8">
+        <v>45841</v>
+      </c>
+      <c r="F72">
+        <v>66</v>
+      </c>
+      <c r="G72">
+        <v>332</v>
+      </c>
+      <c r="H72">
+        <v>326</v>
+      </c>
+      <c r="I72" s="16">
+        <f t="shared" ref="I72:I76" si="3">(B72-B71)/B71</f>
+        <v>4.3477680853732607E-3</v>
+      </c>
+      <c r="J72" s="16">
+        <f>(Processed_US_CA[[#This Row],[Value]]-B60)/B60</f>
+        <v>3.6653791464880932E-3</v>
+      </c>
+      <c r="K72" s="7">
+        <f>Processed_US_CA[[#This Row],[Value]]/B71 * 100</f>
+        <v>100.43477680853732</v>
+      </c>
+      <c r="L72" s="7">
+        <f>Processed_US_CA[[#This Row],[Value]]/B60 * 100</f>
+        <v>100.3665379146488</v>
+      </c>
+      <c r="M72" cm="1">
+        <f t="array" ref="M72">ROUND( Processed_US_CA[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_US_CA[Value], YEAR(Processed_US_CA[Date])=2020) ), 3) * 100</f>
+        <v>129.29999999999998</v>
+      </c>
+      <c r="N72" s="16" cm="1">
+        <f t="array" ref="N72" xml:space="preserve"> Processed_US_CA[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_US_CA[Date], YEAR(Processed_US_CA[Date])=YEAR(Processed_US_CA[[#This Row],[Date]]))), Processed_US_CA[Date], Processed_US_CA[Value]) - 1</f>
+        <v>-6.2749124191762151E-3</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14">
+      <c r="A73" s="6">
+        <f>rawData_HousePriceIndex_US!A73</f>
+        <v>45992</v>
+      </c>
+      <c r="B73" s="21">
+        <f>rawData_HousePriceIndex_US!B73</f>
+        <v>361.20040357866702</v>
+      </c>
+      <c r="C73" t="s">
+        <v>36</v>
+      </c>
+      <c r="E73" s="8"/>
+      <c r="I73" s="16">
+        <f t="shared" si="3"/>
+        <v>1.088492471346011E-3</v>
+      </c>
+      <c r="J73" s="16">
+        <f>(Processed_US_CA[[#This Row],[Value]]-B61)/B61</f>
+        <v>-2.0241216505070586E-3</v>
+      </c>
+      <c r="K73" s="7">
+        <f>Processed_US_CA[[#This Row],[Value]]/B72 * 100</f>
+        <v>100.10884924713459</v>
+      </c>
+      <c r="L73" s="7">
+        <f>Processed_US_CA[[#This Row],[Value]]/B61 * 100</f>
+        <v>99.797587834949297</v>
+      </c>
+      <c r="M73" cm="1">
+        <f t="array" ref="M73">ROUND( Processed_US_CA[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_US_CA[Value], YEAR(Processed_US_CA[Date])=2020) ), 3) * 100</f>
+        <v>129.5</v>
+      </c>
+      <c r="N73" s="16" cm="1">
+        <f t="array" ref="N73" xml:space="preserve"> Processed_US_CA[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_US_CA[Date], YEAR(Processed_US_CA[Date])=YEAR(Processed_US_CA[[#This Row],[Date]]))), Processed_US_CA[Date], Processed_US_CA[Value]) - 1</f>
+        <v>-5.1932501427567335E-3</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14">
+      <c r="A74" s="6">
+        <f>rawData_HousePriceIndex_US!A74</f>
+        <v>46023</v>
+      </c>
+      <c r="B74" s="21">
+        <f>rawData_HousePriceIndex_US!B74</f>
+        <v>360.98095555893298</v>
+      </c>
+      <c r="C74" t="s">
+        <v>36</v>
+      </c>
+      <c r="D74" t="s">
+        <v>22</v>
+      </c>
+      <c r="E74" s="8">
+        <v>45842</v>
+      </c>
+      <c r="F74">
+        <v>66</v>
+      </c>
+      <c r="G74">
+        <v>332</v>
+      </c>
+      <c r="H74">
+        <v>326</v>
+      </c>
+      <c r="I74" s="16">
+        <f t="shared" si="3"/>
+        <v>-6.0755197823651123E-4</v>
+      </c>
+      <c r="J74" s="16">
+        <f>(Processed_US_CA[[#This Row],[Value]]-B62)/B62</f>
+        <v>-5.7976469515955906E-3</v>
+      </c>
+      <c r="K74" s="7">
+        <f>Processed_US_CA[[#This Row],[Value]]/B73 * 100</f>
+        <v>99.939244802176347</v>
+      </c>
+      <c r="L74" s="7">
+        <f>Processed_US_CA[[#This Row],[Value]]/B62 * 100</f>
+        <v>99.420235304840446</v>
+      </c>
+      <c r="M74" cm="1">
+        <f t="array" ref="M74">ROUND( Processed_US_CA[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_US_CA[Value], YEAR(Processed_US_CA[Date])=2020) ), 3) * 100</f>
+        <v>129.4</v>
+      </c>
+      <c r="N74" s="16" cm="1">
+        <f t="array" ref="N74" xml:space="preserve"> Processed_US_CA[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_US_CA[Date], YEAR(Processed_US_CA[Date])=YEAR(Processed_US_CA[[#This Row],[Date]]))), Processed_US_CA[Date], Processed_US_CA[Value]) - 1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14">
+      <c r="A75" s="6">
+        <f>rawData_HousePriceIndex_US!A75</f>
+        <v>46054</v>
+      </c>
+      <c r="B75" s="21">
+        <f>rawData_HousePriceIndex_US!B75</f>
+        <v>361.44834672303</v>
+      </c>
+      <c r="C75" t="s">
+        <v>36</v>
+      </c>
+      <c r="E75" s="8"/>
+      <c r="I75" s="16">
+        <f t="shared" si="3"/>
+        <v>1.2947806716654279E-3</v>
+      </c>
+      <c r="J75" s="16">
+        <f>(Processed_US_CA[[#This Row],[Value]]-B63)/B63</f>
+        <v>-7.1464174618047303E-3</v>
+      </c>
+      <c r="K75" s="7">
+        <f>Processed_US_CA[[#This Row],[Value]]/B74 * 100</f>
+        <v>100.12947806716654</v>
+      </c>
+      <c r="L75" s="7">
+        <f>Processed_US_CA[[#This Row],[Value]]/B63 * 100</f>
+        <v>99.285358253819524</v>
+      </c>
+      <c r="M75" cm="1">
+        <f t="array" ref="M75">ROUND( Processed_US_CA[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_US_CA[Value], YEAR(Processed_US_CA[Date])=2020) ), 3) * 100</f>
+        <v>129.6</v>
+      </c>
+      <c r="N75" s="16" cm="1">
+        <f t="array" ref="N75" xml:space="preserve"> Processed_US_CA[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_US_CA[Date], YEAR(Processed_US_CA[Date])=YEAR(Processed_US_CA[[#This Row],[Date]]))), Processed_US_CA[Date], Processed_US_CA[Value]) - 1</f>
+        <v>1.2947806716654409E-3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14">
+      <c r="A76" s="6">
+        <f>rawData_HousePriceIndex_US!A76</f>
+        <v>46082</v>
+      </c>
+      <c r="B76" s="21">
+        <f>rawData_HousePriceIndex_US!B76</f>
+        <v>360.15886596558403</v>
+      </c>
+      <c r="C76" t="s">
+        <v>36</v>
+      </c>
+      <c r="D76" t="s">
+        <v>22</v>
+      </c>
+      <c r="E76" s="8">
+        <v>45843</v>
+      </c>
+      <c r="F76">
+        <v>66</v>
+      </c>
+      <c r="G76">
+        <v>332</v>
+      </c>
+      <c r="H76">
+        <v>326</v>
+      </c>
+      <c r="I76" s="16">
+        <f t="shared" si="3"/>
+        <v>-3.567538125811578E-3</v>
+      </c>
+      <c r="J76" s="16">
+        <f>(Processed_US_CA[[#This Row],[Value]]-B64)/B64</f>
+        <v>4.7197258480809754E-3</v>
+      </c>
+      <c r="K76" s="7">
+        <f>Processed_US_CA[[#This Row],[Value]]/B75 * 100</f>
+        <v>99.643246187418839</v>
+      </c>
+      <c r="L76" s="7">
+        <f>Processed_US_CA[[#This Row],[Value]]/B64 * 100</f>
+        <v>100.47197258480809</v>
+      </c>
+      <c r="M76" cm="1">
+        <f t="array" ref="M76">ROUND( Processed_US_CA[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_US_CA[Value], YEAR(Processed_US_CA[Date])=2020) ), 3) * 100</f>
+        <v>129.1</v>
+      </c>
+      <c r="N76" s="16" cm="1">
+        <f t="array" ref="N76" xml:space="preserve"> Processed_US_CA[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_US_CA[Date], YEAR(Processed_US_CA[Date])=YEAR(Processed_US_CA[[#This Row],[Date]]))), Processed_US_CA[Date], Processed_US_CA[Value]) - 1</f>
+        <v>-2.2773766335568713E-3</v>
       </c>
     </row>
   </sheetData>
@@ -15894,7 +16969,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B2B3618-7E7D-B043-ACFB-E6824BD3B6F7}">
-  <dimension ref="A1:N71"/>
+  <dimension ref="A1:N77"/>
   <sheetFormatPr defaultColWidth="10.78125" defaultRowHeight="27.5"/>
   <cols>
     <col min="1" max="1" width="9.4765625" bestFit="1" customWidth="1"/>
@@ -19357,32 +20432,32 @@
       </c>
       <c r="B70" s="20">
         <f>rawData_RentPriceIndex_HK!B70</f>
-        <v>200.2</v>
+        <v>199.9</v>
       </c>
       <c r="E70" s="8"/>
       <c r="I70" s="16">
         <f t="shared" si="1"/>
-        <v>1.5007503751875084E-3</v>
+        <v>0</v>
       </c>
       <c r="J70" s="16">
         <f>(Processed_RentPrice_CN_HK__2[[#This Row],[Value]]-B58)/B58</f>
-        <v>2.5089605734766908E-2</v>
+        <v>2.3553507424475137E-2</v>
       </c>
       <c r="K70" s="7">
         <f>Processed_RentPrice_CN_HK__2[[#This Row],[Value]]/B69 * 100</f>
-        <v>100.15007503751876</v>
+        <v>100</v>
       </c>
       <c r="L70" s="7">
         <f>Processed_RentPrice_CN_HK__2[[#This Row],[Value]]/B58 * 100</f>
-        <v>102.5089605734767</v>
+        <v>102.3553507424475</v>
       </c>
       <c r="M70" s="7" cm="1">
         <f t="array" ref="M70">ROUND( Processed_RentPrice_CN_HK__2[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Value], YEAR(Processed_RentPrice_CN_HK__2[Date])=2020) ), 3) * 100</f>
-        <v>111.00000000000001</v>
+        <v>110.9</v>
       </c>
       <c r="N70" s="16" cm="1">
         <f t="array" ref="N70" xml:space="preserve"> Processed_RentPrice_CN_HK__2[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Date], YEAR(Processed_RentPrice_CN_HK__2[Date])=YEAR(Processed_RentPrice_CN_HK__2[[#This Row],[Date]]))), Processed_RentPrice_CN_HK__2[Date], Processed_RentPrice_CN_HK__2[Value]) - 1</f>
-        <v>3.8381742738589075E-2</v>
+        <v>3.6825726141078707E-2</v>
       </c>
     </row>
     <row r="71" spans="1:14">
@@ -19392,7 +20467,7 @@
       </c>
       <c r="B71" s="20">
         <f>rawData_RentPriceIndex_HK!B71</f>
-        <v>200.2</v>
+        <v>199.9</v>
       </c>
       <c r="C71" t="s">
         <v>35</v>
@@ -19413,12 +20488,12 @@
         <v>195</v>
       </c>
       <c r="I71" s="16">
-        <f t="shared" ref="I71" si="2">(B71-B70)/B70</f>
+        <f t="shared" ref="I71:I74" si="2">(B71-B70)/B70</f>
         <v>0</v>
       </c>
       <c r="J71" s="16">
         <f>(Processed_RentPrice_CN_HK__2[[#This Row],[Value]]-B59)/B59</f>
-        <v>3.8920601971977171E-2</v>
+        <v>3.7363777893098173E-2</v>
       </c>
       <c r="K71" s="7">
         <f>Processed_RentPrice_CN_HK__2[[#This Row],[Value]]/B70 * 100</f>
@@ -19426,15 +20501,316 @@
       </c>
       <c r="L71" s="7">
         <f>Processed_RentPrice_CN_HK__2[[#This Row],[Value]]/B59 * 100</f>
-        <v>103.89206019719772</v>
+        <v>103.73637778930981</v>
       </c>
       <c r="M71" s="7" cm="1">
         <f t="array" ref="M71">ROUND( Processed_RentPrice_CN_HK__2[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Value], YEAR(Processed_RentPrice_CN_HK__2[Date])=2020) ), 3) * 100</f>
-        <v>111.00000000000001</v>
+        <v>110.9</v>
       </c>
       <c r="N71" s="16" cm="1">
         <f t="array" ref="N71" xml:space="preserve"> Processed_RentPrice_CN_HK__2[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Date], YEAR(Processed_RentPrice_CN_HK__2[Date])=YEAR(Processed_RentPrice_CN_HK__2[[#This Row],[Date]]))), Processed_RentPrice_CN_HK__2[Date], Processed_RentPrice_CN_HK__2[Value]) - 1</f>
-        <v>3.8381742738589075E-2</v>
+        <v>3.6825726141078707E-2</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14">
+      <c r="A72" s="18">
+        <f>rawData_RentPriceIndex_HK!A72</f>
+        <v>45962</v>
+      </c>
+      <c r="B72" s="20">
+        <f>rawData_RentPriceIndex_HK!B72</f>
+        <v>200.4</v>
+      </c>
+      <c r="C72" t="s">
+        <v>35</v>
+      </c>
+      <c r="D72" t="s">
+        <v>22</v>
+      </c>
+      <c r="E72" s="8">
+        <v>45839</v>
+      </c>
+      <c r="F72">
+        <v>67.428571428571402</v>
+      </c>
+      <c r="G72">
+        <v>196</v>
+      </c>
+      <c r="H72">
+        <v>195.42857142857099</v>
+      </c>
+      <c r="I72" s="16">
+        <f t="shared" si="2"/>
+        <v>2.5012506253126563E-3</v>
+      </c>
+      <c r="J72" s="16">
+        <f>(Processed_RentPrice_CN_HK__2[[#This Row],[Value]]-B60)/B60</f>
+        <v>4.4293903074517978E-2</v>
+      </c>
+      <c r="K72" s="7">
+        <f>Processed_RentPrice_CN_HK__2[[#This Row],[Value]]/B71 * 100</f>
+        <v>100.25012506253125</v>
+      </c>
+      <c r="L72" s="7">
+        <f>Processed_RentPrice_CN_HK__2[[#This Row],[Value]]/B60 * 100</f>
+        <v>104.4293903074518</v>
+      </c>
+      <c r="M72" s="7" cm="1">
+        <f t="array" ref="M72">ROUND( Processed_RentPrice_CN_HK__2[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Value], YEAR(Processed_RentPrice_CN_HK__2[Date])=2020) ), 3) * 100</f>
+        <v>111.1</v>
+      </c>
+      <c r="N72" s="16" cm="1">
+        <f t="array" ref="N72" xml:space="preserve"> Processed_RentPrice_CN_HK__2[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Date], YEAR(Processed_RentPrice_CN_HK__2[Date])=YEAR(Processed_RentPrice_CN_HK__2[[#This Row],[Date]]))), Processed_RentPrice_CN_HK__2[Date], Processed_RentPrice_CN_HK__2[Value]) - 1</f>
+        <v>3.9419087136929321E-2</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14">
+      <c r="A73" s="18">
+        <f>rawData_RentPriceIndex_HK!A73</f>
+        <v>45992</v>
+      </c>
+      <c r="B73" s="20">
+        <f>rawData_RentPriceIndex_HK!B73</f>
+        <v>200.4</v>
+      </c>
+      <c r="C73" t="s">
+        <v>35</v>
+      </c>
+      <c r="D73" t="s">
+        <v>22</v>
+      </c>
+      <c r="E73" s="8">
+        <v>45870</v>
+      </c>
+      <c r="F73">
+        <v>67.714285714285694</v>
+      </c>
+      <c r="G73">
+        <v>196</v>
+      </c>
+      <c r="H73">
+        <v>195.71428571428601</v>
+      </c>
+      <c r="I73" s="16">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="J73" s="16">
+        <f>(Processed_RentPrice_CN_HK__2[[#This Row],[Value]]-B61)/B61</f>
+        <v>4.1038961038961069E-2</v>
+      </c>
+      <c r="K73" s="7">
+        <f>Processed_RentPrice_CN_HK__2[[#This Row],[Value]]/B72 * 100</f>
+        <v>100</v>
+      </c>
+      <c r="L73" s="7">
+        <f>Processed_RentPrice_CN_HK__2[[#This Row],[Value]]/B61 * 100</f>
+        <v>104.1038961038961</v>
+      </c>
+      <c r="M73" s="7" cm="1">
+        <f t="array" ref="M73">ROUND( Processed_RentPrice_CN_HK__2[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Value], YEAR(Processed_RentPrice_CN_HK__2[Date])=2020) ), 3) * 100</f>
+        <v>111.1</v>
+      </c>
+      <c r="N73" s="16" cm="1">
+        <f t="array" ref="N73" xml:space="preserve"> Processed_RentPrice_CN_HK__2[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Date], YEAR(Processed_RentPrice_CN_HK__2[Date])=YEAR(Processed_RentPrice_CN_HK__2[[#This Row],[Date]]))), Processed_RentPrice_CN_HK__2[Date], Processed_RentPrice_CN_HK__2[Value]) - 1</f>
+        <v>3.9419087136929321E-2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14">
+      <c r="A74" s="18">
+        <f>rawData_RentPriceIndex_HK!A74</f>
+        <v>46023</v>
+      </c>
+      <c r="B74" s="20">
+        <f>rawData_RentPriceIndex_HK!B74</f>
+        <v>200.8</v>
+      </c>
+      <c r="E74" s="8"/>
+      <c r="F74">
+        <v>68</v>
+      </c>
+      <c r="H74">
+        <v>196</v>
+      </c>
+      <c r="I74" s="16">
+        <f t="shared" si="2"/>
+        <v>1.9960079840319646E-3</v>
+      </c>
+      <c r="J74" s="16">
+        <f>(Processed_RentPrice_CN_HK__2[[#This Row],[Value]]-B62)/B62</f>
+        <v>4.1493775933609957E-2</v>
+      </c>
+      <c r="K74" s="7">
+        <f>Processed_RentPrice_CN_HK__2[[#This Row],[Value]]/B73 * 100</f>
+        <v>100.1996007984032</v>
+      </c>
+      <c r="L74" s="7">
+        <f>Processed_RentPrice_CN_HK__2[[#This Row],[Value]]/B62 * 100</f>
+        <v>104.14937759336101</v>
+      </c>
+      <c r="M74" s="7" cm="1">
+        <f t="array" ref="M74">ROUND( Processed_RentPrice_CN_HK__2[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Value], YEAR(Processed_RentPrice_CN_HK__2[Date])=2020) ), 3) * 100</f>
+        <v>111.4</v>
+      </c>
+      <c r="N74" s="16" cm="1">
+        <f t="array" ref="N74" xml:space="preserve"> Processed_RentPrice_CN_HK__2[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Date], YEAR(Processed_RentPrice_CN_HK__2[Date])=YEAR(Processed_RentPrice_CN_HK__2[[#This Row],[Date]]))), Processed_RentPrice_CN_HK__2[Date], Processed_RentPrice_CN_HK__2[Value]) - 1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14">
+      <c r="A75" s="18">
+        <f>rawData_RentPriceIndex_HK!A75</f>
+        <v>46054</v>
+      </c>
+      <c r="B75" s="20">
+        <f>rawData_RentPriceIndex_HK!B75</f>
+        <v>201</v>
+      </c>
+      <c r="C75" t="s">
+        <v>35</v>
+      </c>
+      <c r="D75" t="s">
+        <v>22</v>
+      </c>
+      <c r="E75" s="8">
+        <v>45871</v>
+      </c>
+      <c r="F75">
+        <v>68.285714285714306</v>
+      </c>
+      <c r="G75">
+        <v>196</v>
+      </c>
+      <c r="H75">
+        <v>196.28571428571399</v>
+      </c>
+      <c r="I75" s="16">
+        <f t="shared" ref="I75:I76" si="3">(B75-B74)/B74</f>
+        <v>9.9601593625492347E-4</v>
+      </c>
+      <c r="J75" s="16">
+        <f>(Processed_RentPrice_CN_HK__2[[#This Row],[Value]]-B63)/B63</f>
+        <v>4.145077720207254E-2</v>
+      </c>
+      <c r="K75" s="7">
+        <f>Processed_RentPrice_CN_HK__2[[#This Row],[Value]]/B74 * 100</f>
+        <v>100.09960159362549</v>
+      </c>
+      <c r="L75" s="7">
+        <f>Processed_RentPrice_CN_HK__2[[#This Row],[Value]]/B63 * 100</f>
+        <v>104.14507772020724</v>
+      </c>
+      <c r="M75" s="7" cm="1">
+        <f t="array" ref="M75">ROUND( Processed_RentPrice_CN_HK__2[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Value], YEAR(Processed_RentPrice_CN_HK__2[Date])=2020) ), 3) * 100</f>
+        <v>111.5</v>
+      </c>
+      <c r="N75" s="16" cm="1">
+        <f t="array" ref="N75" xml:space="preserve"> Processed_RentPrice_CN_HK__2[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Date], YEAR(Processed_RentPrice_CN_HK__2[Date])=YEAR(Processed_RentPrice_CN_HK__2[[#This Row],[Date]]))), Processed_RentPrice_CN_HK__2[Date], Processed_RentPrice_CN_HK__2[Value]) - 1</f>
+        <v>9.960159362549792E-4</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14">
+      <c r="A76" s="18">
+        <f>rawData_RentPriceIndex_HK!A76</f>
+        <v>46082</v>
+      </c>
+      <c r="B76" s="20">
+        <f>rawData_RentPriceIndex_HK!B76</f>
+        <v>202.2</v>
+      </c>
+      <c r="C76" t="s">
+        <v>35</v>
+      </c>
+      <c r="D76" t="s">
+        <v>22</v>
+      </c>
+      <c r="E76" s="8">
+        <v>45839</v>
+      </c>
+      <c r="F76">
+        <v>68.571428571428598</v>
+      </c>
+      <c r="G76">
+        <v>196</v>
+      </c>
+      <c r="H76">
+        <v>196.57142857142901</v>
+      </c>
+      <c r="I76" s="16">
+        <f t="shared" si="3"/>
+        <v>5.970149253731287E-3</v>
+      </c>
+      <c r="J76" s="16">
+        <f>(Processed_RentPrice_CN_HK__2[[#This Row],[Value]]-B64)/B64</f>
+        <v>4.7125841532884488E-2</v>
+      </c>
+      <c r="K76" s="7">
+        <f>Processed_RentPrice_CN_HK__2[[#This Row],[Value]]/B75 * 100</f>
+        <v>100.59701492537312</v>
+      </c>
+      <c r="L76" s="7">
+        <f>Processed_RentPrice_CN_HK__2[[#This Row],[Value]]/B64 * 100</f>
+        <v>104.71258415328846</v>
+      </c>
+      <c r="M76" s="7" cm="1">
+        <f t="array" ref="M76">ROUND( Processed_RentPrice_CN_HK__2[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Value], YEAR(Processed_RentPrice_CN_HK__2[Date])=2020) ), 3) * 100</f>
+        <v>112.1</v>
+      </c>
+      <c r="N76" s="16" cm="1">
+        <f t="array" ref="N76" xml:space="preserve"> Processed_RentPrice_CN_HK__2[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Date], YEAR(Processed_RentPrice_CN_HK__2[Date])=YEAR(Processed_RentPrice_CN_HK__2[[#This Row],[Date]]))), Processed_RentPrice_CN_HK__2[Date], Processed_RentPrice_CN_HK__2[Value]) - 1</f>
+        <v>6.9721115537848544E-3</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14">
+      <c r="A77" s="18">
+        <f>rawData_RentPriceIndex_HK!A77</f>
+        <v>46113</v>
+      </c>
+      <c r="B77" s="20">
+        <f>rawData_RentPriceIndex_HK!B77</f>
+        <v>203.4</v>
+      </c>
+      <c r="C77" t="s">
+        <v>35</v>
+      </c>
+      <c r="D77" t="s">
+        <v>22</v>
+      </c>
+      <c r="E77" s="8">
+        <v>45807</v>
+      </c>
+      <c r="F77">
+        <v>68.857142857142904</v>
+      </c>
+      <c r="G77">
+        <v>196</v>
+      </c>
+      <c r="H77">
+        <v>196.857142857144</v>
+      </c>
+      <c r="I77" s="16">
+        <f t="shared" ref="I77" si="4">(B77-B76)/B76</f>
+        <v>5.9347181008902921E-3</v>
+      </c>
+      <c r="J77" s="16">
+        <f>(Processed_RentPrice_CN_HK__2[[#This Row],[Value]]-B65)/B65</f>
+        <v>4.899432697266632E-2</v>
+      </c>
+      <c r="K77" s="7">
+        <f>Processed_RentPrice_CN_HK__2[[#This Row],[Value]]/B76 * 100</f>
+        <v>100.59347181008901</v>
+      </c>
+      <c r="L77" s="7">
+        <f>Processed_RentPrice_CN_HK__2[[#This Row],[Value]]/B65 * 100</f>
+        <v>104.89943269726663</v>
+      </c>
+      <c r="M77" s="7" cm="1">
+        <f t="array" ref="M77">ROUND( Processed_RentPrice_CN_HK__2[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Value], YEAR(Processed_RentPrice_CN_HK__2[Date])=2020) ), 3) * 100</f>
+        <v>112.79999999999998</v>
+      </c>
+      <c r="N77" s="16" cm="1">
+        <f t="array" ref="N77" xml:space="preserve"> Processed_RentPrice_CN_HK__2[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_RentPrice_CN_HK__2[Date], YEAR(Processed_RentPrice_CN_HK__2[Date])=YEAR(Processed_RentPrice_CN_HK__2[[#This Row],[Date]]))), Processed_RentPrice_CN_HK__2[Date], Processed_RentPrice_CN_HK__2[Value]) - 1</f>
+        <v>1.294820717131473E-2</v>
       </c>
     </row>
   </sheetData>
@@ -19449,7 +20825,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{959DEF48-451F-8141-B290-384BA45A03F2}">
-  <dimension ref="A1:N70"/>
+  <dimension ref="A1:N77"/>
   <sheetFormatPr defaultColWidth="10.78125" defaultRowHeight="27.5"/>
   <cols>
     <col min="1" max="1" width="9.4765625" bestFit="1" customWidth="1"/>
@@ -22828,7 +24204,7 @@
         <v>506</v>
       </c>
       <c r="I68" s="16">
-        <f t="shared" ref="I68:I70" si="1">(B68-B67)/B67</f>
+        <f t="shared" ref="I68:I71" si="1">(B68-B67)/B67</f>
         <v>-1.7191293081706106E-3</v>
       </c>
       <c r="J68" s="16">
@@ -22937,6 +24313,353 @@
       <c r="N70" s="16" cm="1">
         <f t="array" ref="N70" xml:space="preserve"> Processed_RentPrice_US_CA__2[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_RentPrice_US_CA__2[Date], YEAR(Processed_RentPrice_US_CA__2[Date])=YEAR(Processed_RentPrice_US_CA__2[[#This Row],[Date]]))), Processed_RentPrice_US_CA__2[Date], Processed_RentPrice_US_CA__2[Value]) - 1</f>
         <v>7.3341177516175193E-3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14">
+      <c r="A71" s="8">
+        <f>rawData_RentPriceIndex_US!A71</f>
+        <v>45931</v>
+      </c>
+      <c r="B71">
+        <f>rawData_RentPriceIndex_US!B71</f>
+        <v>521.37699999999995</v>
+      </c>
+      <c r="C71" t="s">
+        <v>35</v>
+      </c>
+      <c r="D71" t="s">
+        <v>22</v>
+      </c>
+      <c r="E71" s="8">
+        <v>45901</v>
+      </c>
+      <c r="F71">
+        <v>68</v>
+      </c>
+      <c r="G71">
+        <v>519.66666666666697</v>
+      </c>
+      <c r="H71">
+        <v>510.66666666666703</v>
+      </c>
+      <c r="I71" s="16">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J71" s="16">
+        <f>(Processed_RentPrice_US_CA__2[[#This Row],[Value]]-B59)/B59</f>
+        <v>1.6761508789309907E-2</v>
+      </c>
+      <c r="K71" s="7">
+        <f>Processed_RentPrice_US_CA__2[[#This Row],[Value]]/B70 * 100</f>
+        <v>100</v>
+      </c>
+      <c r="L71" s="7">
+        <f>Processed_RentPrice_US_CA__2[[#This Row],[Value]]/B59 * 100</f>
+        <v>101.67615087893098</v>
+      </c>
+      <c r="M71" cm="1">
+        <f t="array" ref="M71">ROUND( Processed_RentPrice_US_CA__2[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_RentPrice_US_CA__2[Value], YEAR(Processed_RentPrice_US_CA__2[Date])=2020) ), 3) * 100</f>
+        <v>111.60000000000001</v>
+      </c>
+      <c r="N71" s="16" cm="1">
+        <f t="array" ref="N71" xml:space="preserve"> Processed_RentPrice_US_CA__2[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_RentPrice_US_CA__2[Date], YEAR(Processed_RentPrice_US_CA__2[Date])=YEAR(Processed_RentPrice_US_CA__2[[#This Row],[Date]]))), Processed_RentPrice_US_CA__2[Date], Processed_RentPrice_US_CA__2[Value]) - 1</f>
+        <v>7.3341177516175193E-3</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14">
+      <c r="A72" s="8">
+        <f>rawData_RentPriceIndex_US!A72</f>
+        <v>45962</v>
+      </c>
+      <c r="B72">
+        <f>rawData_RentPriceIndex_US!B72</f>
+        <v>522.02599999999995</v>
+      </c>
+      <c r="C72" t="s">
+        <v>35</v>
+      </c>
+      <c r="D72" t="s">
+        <v>22</v>
+      </c>
+      <c r="E72" s="8">
+        <v>45931</v>
+      </c>
+      <c r="F72">
+        <v>69</v>
+      </c>
+      <c r="G72">
+        <v>520.16666666666697</v>
+      </c>
+      <c r="H72">
+        <v>512.66666666666697</v>
+      </c>
+      <c r="I72" s="16">
+        <f t="shared" ref="I72:I77" si="2">(B72-B71)/B71</f>
+        <v>1.2447806481682179E-3</v>
+      </c>
+      <c r="J72" s="16">
+        <f>(Processed_RentPrice_US_CA__2[[#This Row],[Value]]-B60)/B60</f>
+        <v>1.6615578760413804E-2</v>
+      </c>
+      <c r="K72" s="7">
+        <f>Processed_RentPrice_US_CA__2[[#This Row],[Value]]/B71 * 100</f>
+        <v>100.12447806481681</v>
+      </c>
+      <c r="L72" s="7">
+        <f>Processed_RentPrice_US_CA__2[[#This Row],[Value]]/B60 * 100</f>
+        <v>101.66155787604139</v>
+      </c>
+      <c r="M72" cm="1">
+        <f t="array" ref="M72">ROUND( Processed_RentPrice_US_CA__2[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_RentPrice_US_CA__2[Value], YEAR(Processed_RentPrice_US_CA__2[Date])=2020) ), 3) * 100</f>
+        <v>111.80000000000001</v>
+      </c>
+      <c r="N72" s="16" cm="1">
+        <f t="array" ref="N72" xml:space="preserve"> Processed_RentPrice_US_CA__2[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_RentPrice_US_CA__2[Date], YEAR(Processed_RentPrice_US_CA__2[Date])=YEAR(Processed_RentPrice_US_CA__2[[#This Row],[Date]]))), Processed_RentPrice_US_CA__2[Date], Processed_RentPrice_US_CA__2[Value]) - 1</f>
+        <v>8.588027767634232E-3</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14">
+      <c r="A73" s="8">
+        <f>rawData_RentPriceIndex_US!A73</f>
+        <v>45992</v>
+      </c>
+      <c r="B73">
+        <f>rawData_RentPriceIndex_US!B73</f>
+        <v>524.77700000000004</v>
+      </c>
+      <c r="C73" t="s">
+        <v>35</v>
+      </c>
+      <c r="D73" t="s">
+        <v>22</v>
+      </c>
+      <c r="E73" s="8">
+        <v>45962</v>
+      </c>
+      <c r="F73">
+        <v>70</v>
+      </c>
+      <c r="G73">
+        <v>520.66666666666697</v>
+      </c>
+      <c r="H73">
+        <v>514.66666666666697</v>
+      </c>
+      <c r="I73" s="16">
+        <f t="shared" si="2"/>
+        <v>5.2698524594562155E-3</v>
+      </c>
+      <c r="J73" s="16">
+        <f>(Processed_RentPrice_US_CA__2[[#This Row],[Value]]-B61)/B61</f>
+        <v>1.7234427761172191E-2</v>
+      </c>
+      <c r="K73" s="7">
+        <f>Processed_RentPrice_US_CA__2[[#This Row],[Value]]/B72 * 100</f>
+        <v>100.52698524594564</v>
+      </c>
+      <c r="L73" s="7">
+        <f>Processed_RentPrice_US_CA__2[[#This Row],[Value]]/B61 * 100</f>
+        <v>101.72344277611722</v>
+      </c>
+      <c r="M73" cm="1">
+        <f t="array" ref="M73">ROUND( Processed_RentPrice_US_CA__2[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_RentPrice_US_CA__2[Value], YEAR(Processed_RentPrice_US_CA__2[Date])=2020) ), 3) * 100</f>
+        <v>112.4</v>
+      </c>
+      <c r="N73" s="16" cm="1">
+        <f t="array" ref="N73" xml:space="preserve"> Processed_RentPrice_US_CA__2[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_RentPrice_US_CA__2[Date], YEAR(Processed_RentPrice_US_CA__2[Date])=YEAR(Processed_RentPrice_US_CA__2[[#This Row],[Date]]))), Processed_RentPrice_US_CA__2[Date], Processed_RentPrice_US_CA__2[Value]) - 1</f>
+        <v>1.3903137866343673E-2</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14">
+      <c r="A74" s="8">
+        <f>rawData_RentPriceIndex_US!A74</f>
+        <v>46023</v>
+      </c>
+      <c r="B74">
+        <f>rawData_RentPriceIndex_US!B74</f>
+        <v>526.399</v>
+      </c>
+      <c r="E74" s="8"/>
+      <c r="I74" s="16">
+        <f t="shared" si="2"/>
+        <v>3.0908366791988925E-3</v>
+      </c>
+      <c r="J74" s="16">
+        <f>(Processed_RentPrice_US_CA__2[[#This Row],[Value]]-B62)/B62</f>
+        <v>1.7036946874015822E-2</v>
+      </c>
+      <c r="K74" s="7">
+        <f>Processed_RentPrice_US_CA__2[[#This Row],[Value]]/B73 * 100</f>
+        <v>100.30908366791988</v>
+      </c>
+      <c r="L74" s="7">
+        <f>Processed_RentPrice_US_CA__2[[#This Row],[Value]]/B62 * 100</f>
+        <v>101.70369468740159</v>
+      </c>
+      <c r="M74" cm="1">
+        <f t="array" ref="M74">ROUND( Processed_RentPrice_US_CA__2[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_RentPrice_US_CA__2[Value], YEAR(Processed_RentPrice_US_CA__2[Date])=2020) ), 3) * 100</f>
+        <v>112.7</v>
+      </c>
+      <c r="N74" s="16" cm="1">
+        <f t="array" ref="N74" xml:space="preserve"> Processed_RentPrice_US_CA__2[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_RentPrice_US_CA__2[Date], YEAR(Processed_RentPrice_US_CA__2[Date])=YEAR(Processed_RentPrice_US_CA__2[[#This Row],[Date]]))), Processed_RentPrice_US_CA__2[Date], Processed_RentPrice_US_CA__2[Value]) - 1</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14">
+      <c r="A75" s="8">
+        <f>rawData_RentPriceIndex_US!A75</f>
+        <v>46054</v>
+      </c>
+      <c r="B75">
+        <f>rawData_RentPriceIndex_US!B75</f>
+        <v>527.20100000000002</v>
+      </c>
+      <c r="C75" t="s">
+        <v>35</v>
+      </c>
+      <c r="D75" t="s">
+        <v>22</v>
+      </c>
+      <c r="E75" s="8">
+        <v>45992</v>
+      </c>
+      <c r="F75">
+        <v>71</v>
+      </c>
+      <c r="G75">
+        <v>521.16666666666697</v>
+      </c>
+      <c r="H75">
+        <v>516.66666666666697</v>
+      </c>
+      <c r="I75" s="16">
+        <f t="shared" si="2"/>
+        <v>1.5235591253023293E-3</v>
+      </c>
+      <c r="J75" s="16">
+        <f>(Processed_RentPrice_US_CA__2[[#This Row],[Value]]-B63)/B63</f>
+        <v>1.9370319596738541E-2</v>
+      </c>
+      <c r="K75" s="7">
+        <f>Processed_RentPrice_US_CA__2[[#This Row],[Value]]/B74 * 100</f>
+        <v>100.15235591253023</v>
+      </c>
+      <c r="L75" s="7">
+        <f>Processed_RentPrice_US_CA__2[[#This Row],[Value]]/B63 * 100</f>
+        <v>101.93703195967385</v>
+      </c>
+      <c r="M75" cm="1">
+        <f t="array" ref="M75">ROUND( Processed_RentPrice_US_CA__2[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_RentPrice_US_CA__2[Value], YEAR(Processed_RentPrice_US_CA__2[Date])=2020) ), 3) * 100</f>
+        <v>112.9</v>
+      </c>
+      <c r="N75" s="16" cm="1">
+        <f t="array" ref="N75" xml:space="preserve"> Processed_RentPrice_US_CA__2[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_RentPrice_US_CA__2[Date], YEAR(Processed_RentPrice_US_CA__2[Date])=YEAR(Processed_RentPrice_US_CA__2[[#This Row],[Date]]))), Processed_RentPrice_US_CA__2[Date], Processed_RentPrice_US_CA__2[Value]) - 1</f>
+        <v>1.5235591253022207E-3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14">
+      <c r="A76" s="8">
+        <f>rawData_RentPriceIndex_US!A76</f>
+        <v>46082</v>
+      </c>
+      <c r="B76">
+        <f>rawData_RentPriceIndex_US!B76</f>
+        <v>528.14700000000005</v>
+      </c>
+      <c r="C76" t="s">
+        <v>35</v>
+      </c>
+      <c r="D76" t="s">
+        <v>22</v>
+      </c>
+      <c r="E76" s="8">
+        <v>46023</v>
+      </c>
+      <c r="F76">
+        <v>72</v>
+      </c>
+      <c r="G76">
+        <v>521.66666666666697</v>
+      </c>
+      <c r="H76">
+        <v>518.66666666666697</v>
+      </c>
+      <c r="I76" s="16">
+        <f t="shared" si="2"/>
+        <v>1.7943820288657008E-3</v>
+      </c>
+      <c r="J76" s="16">
+        <f>(Processed_RentPrice_US_CA__2[[#This Row],[Value]]-B64)/B64</f>
+        <v>1.8619344909188738E-2</v>
+      </c>
+      <c r="K76" s="7">
+        <f>Processed_RentPrice_US_CA__2[[#This Row],[Value]]/B75 * 100</f>
+        <v>100.17943820288657</v>
+      </c>
+      <c r="L76" s="7">
+        <f>Processed_RentPrice_US_CA__2[[#This Row],[Value]]/B64 * 100</f>
+        <v>101.86193449091887</v>
+      </c>
+      <c r="M76" cm="1">
+        <f t="array" ref="M76">ROUND( Processed_RentPrice_US_CA__2[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_RentPrice_US_CA__2[Value], YEAR(Processed_RentPrice_US_CA__2[Date])=2020) ), 3) * 100</f>
+        <v>113.1</v>
+      </c>
+      <c r="N76" s="16" cm="1">
+        <f t="array" ref="N76" xml:space="preserve"> Processed_RentPrice_US_CA__2[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_RentPrice_US_CA__2[Date], YEAR(Processed_RentPrice_US_CA__2[Date])=YEAR(Processed_RentPrice_US_CA__2[[#This Row],[Date]]))), Processed_RentPrice_US_CA__2[Date], Processed_RentPrice_US_CA__2[Value]) - 1</f>
+        <v>3.3206750012824138E-3</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14">
+      <c r="A77" s="8">
+        <f>rawData_RentPriceIndex_US!A77</f>
+        <v>46113</v>
+      </c>
+      <c r="B77">
+        <f>rawData_RentPriceIndex_US!B77</f>
+        <v>532.15300000000002</v>
+      </c>
+      <c r="C77" t="s">
+        <v>35</v>
+      </c>
+      <c r="D77" t="s">
+        <v>22</v>
+      </c>
+      <c r="E77" s="8">
+        <v>46054</v>
+      </c>
+      <c r="F77">
+        <v>73</v>
+      </c>
+      <c r="G77">
+        <v>522.16666666666697</v>
+      </c>
+      <c r="H77">
+        <v>520.66666666666697</v>
+      </c>
+      <c r="I77" s="16">
+        <f t="shared" si="2"/>
+        <v>7.5850094765282606E-3</v>
+      </c>
+      <c r="J77" s="16">
+        <f>(Processed_RentPrice_US_CA__2[[#This Row],[Value]]-B65)/B65</f>
+        <v>2.6597037614349773E-2</v>
+      </c>
+      <c r="K77" s="7">
+        <f>Processed_RentPrice_US_CA__2[[#This Row],[Value]]/B76 * 100</f>
+        <v>100.75850094765282</v>
+      </c>
+      <c r="L77" s="7">
+        <f>Processed_RentPrice_US_CA__2[[#This Row],[Value]]/B65 * 100</f>
+        <v>102.65970376143498</v>
+      </c>
+      <c r="M77" cm="1">
+        <f t="array" ref="M77">ROUND( Processed_RentPrice_US_CA__2[[#This Row],[Value]] / AVERAGE( _xlfn._xlws.FILTER(Processed_RentPrice_US_CA__2[Value], YEAR(Processed_RentPrice_US_CA__2[Date])=2020) ), 3) * 100</f>
+        <v>113.9</v>
+      </c>
+      <c r="N77" s="16" cm="1">
+        <f t="array" ref="N77" xml:space="preserve"> Processed_RentPrice_US_CA__2[[#This Row],[Value]] / _xlfn.XLOOKUP(MIN(_xlfn._xlws.FILTER(Processed_RentPrice_US_CA__2[Date], YEAR(Processed_RentPrice_US_CA__2[Date])=YEAR(Processed_RentPrice_US_CA__2[[#This Row],[Date]]))), Processed_RentPrice_US_CA__2[Date], Processed_RentPrice_US_CA__2[Value]) - 1</f>
+        <v>1.0930871829163857E-2</v>
       </c>
     </row>
   </sheetData>
@@ -22951,7 +24674,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{319ACA72-8BFE-AE41-A63E-49ECCE7478F1}">
-  <dimension ref="A1:E73"/>
+  <dimension ref="A1:E79"/>
   <sheetFormatPr defaultColWidth="10.78125" defaultRowHeight="27.5"/>
   <cols>
     <col min="1" max="1" width="10.5625" style="6"/>
@@ -24188,7 +25911,7 @@
         <v>45992</v>
       </c>
       <c r="B73" s="7">
-        <v>53601</v>
+        <v>53357</v>
       </c>
       <c r="C73" t="s">
         <v>25</v>
@@ -24198,6 +25921,108 @@
       </c>
       <c r="E73" s="5">
         <v>45992</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
+      <c r="A74" s="6">
+        <v>46023</v>
+      </c>
+      <c r="B74" s="7">
+        <v>53390</v>
+      </c>
+      <c r="C74" t="s">
+        <v>25</v>
+      </c>
+      <c r="D74" t="s">
+        <v>23</v>
+      </c>
+      <c r="E74" s="5">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
+      <c r="A75" s="6">
+        <v>46054</v>
+      </c>
+      <c r="B75" s="7">
+        <v>53781</v>
+      </c>
+      <c r="C75" t="s">
+        <v>25</v>
+      </c>
+      <c r="D75" t="s">
+        <v>23</v>
+      </c>
+      <c r="E75" s="5">
+        <v>46054</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5">
+      <c r="A76" s="6">
+        <v>46082</v>
+      </c>
+      <c r="B76" s="7">
+        <v>53598</v>
+      </c>
+      <c r="C76" t="s">
+        <v>25</v>
+      </c>
+      <c r="D76" t="s">
+        <v>23</v>
+      </c>
+      <c r="E76" s="5">
+        <v>46082</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5">
+      <c r="A77" s="6">
+        <v>46113</v>
+      </c>
+      <c r="B77" s="7">
+        <v>53066</v>
+      </c>
+      <c r="C77" t="s">
+        <v>25</v>
+      </c>
+      <c r="D77" t="s">
+        <v>23</v>
+      </c>
+      <c r="E77" s="5">
+        <v>46113</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5">
+      <c r="A78" s="6">
+        <v>46143</v>
+      </c>
+      <c r="B78" s="7">
+        <v>52386</v>
+      </c>
+      <c r="C78" t="s">
+        <v>25</v>
+      </c>
+      <c r="D78" t="s">
+        <v>23</v>
+      </c>
+      <c r="E78" s="5">
+        <v>46143</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5">
+      <c r="A79" s="6">
+        <v>46174</v>
+      </c>
+      <c r="B79" s="7">
+        <v>52253</v>
+      </c>
+      <c r="C79" t="s">
+        <v>25</v>
+      </c>
+      <c r="D79" t="s">
+        <v>23</v>
+      </c>
+      <c r="E79" s="5">
+        <v>46174</v>
       </c>
     </row>
   </sheetData>
@@ -24209,7 +26034,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8351C2C8-E9AB-B94B-942F-9219AC52EAE5}">
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr defaultColWidth="10.78125" defaultRowHeight="27.5"/>
   <cols>
     <col min="1" max="1" width="10.5625" style="6"/>
@@ -25394,8 +27219,8 @@
       <c r="A70" s="6">
         <v>45901</v>
       </c>
-      <c r="B70" s="10">
-        <v>293.10000000000002</v>
+      <c r="B70">
+        <v>293.39999999999998</v>
       </c>
       <c r="C70" t="s">
         <v>28</v>
@@ -25411,8 +27236,8 @@
       <c r="A71" s="6">
         <v>45931</v>
       </c>
-      <c r="B71" s="10">
-        <v>294.3</v>
+      <c r="B71">
+        <v>294.89999999999998</v>
       </c>
       <c r="C71" t="s">
         <v>28</v>
@@ -25422,6 +27247,108 @@
       </c>
       <c r="E71" s="6">
         <v>45931</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5">
+      <c r="A72" s="6">
+        <v>45962</v>
+      </c>
+      <c r="B72">
+        <v>298.7</v>
+      </c>
+      <c r="C72" t="s">
+        <v>28</v>
+      </c>
+      <c r="D72" t="s">
+        <v>23</v>
+      </c>
+      <c r="E72" s="6">
+        <v>45962</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5">
+      <c r="A73" s="6">
+        <v>45992</v>
+      </c>
+      <c r="B73">
+        <v>299.60000000000002</v>
+      </c>
+      <c r="C73" t="s">
+        <v>28</v>
+      </c>
+      <c r="D73" t="s">
+        <v>23</v>
+      </c>
+      <c r="E73" s="6">
+        <v>45992</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
+      <c r="A74" s="6">
+        <v>46023</v>
+      </c>
+      <c r="B74">
+        <v>303</v>
+      </c>
+      <c r="C74" t="s">
+        <v>28</v>
+      </c>
+      <c r="D74" t="s">
+        <v>23</v>
+      </c>
+      <c r="E74" s="6">
+        <v>46023</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
+      <c r="A75" s="6">
+        <v>46054</v>
+      </c>
+      <c r="B75">
+        <v>308.5</v>
+      </c>
+      <c r="C75" t="s">
+        <v>28</v>
+      </c>
+      <c r="D75" t="s">
+        <v>23</v>
+      </c>
+      <c r="E75" s="6">
+        <v>46054</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5">
+      <c r="A76" s="6">
+        <v>46082</v>
+      </c>
+      <c r="B76">
+        <v>312.8</v>
+      </c>
+      <c r="C76" t="s">
+        <v>28</v>
+      </c>
+      <c r="D76" t="s">
+        <v>23</v>
+      </c>
+      <c r="E76" s="6">
+        <v>46082</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5">
+      <c r="A77" s="6">
+        <v>46113</v>
+      </c>
+      <c r="B77">
+        <v>316.60000000000002</v>
+      </c>
+      <c r="C77" t="s">
+        <v>28</v>
+      </c>
+      <c r="D77" t="s">
+        <v>23</v>
+      </c>
+      <c r="E77" s="6">
+        <v>46113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>